<commit_message>
Publish remaining workbook and site updates
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Final-All-Under-10-Review.xlsx
+++ b/Final-All-Under-10-Review.xlsx
@@ -1,18 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC43EB3-5BC8-4661-A59E-76495FEDC9A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="All Stocks" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Stocks under 10Rs" state="visible" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
+    <sheet name="All Stocks" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3719" uniqueCount="2226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3725" uniqueCount="2245">
   <si>
     <t>Sector</t>
   </si>
@@ -6689,34 +6693,291 @@
     <t>https://www.screener.in/company/539040/</t>
   </si>
   <si>
-    <t>No verified stocks matched. Pledged percentage &lt; 0 is not a valid no-pledge filter; use 0% for no pledged shares.</t>
+    <t>Healthcare</t>
+  </si>
+  <si>
+    <r>
+      <t>Pharmaceuticals</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +14%, ROCE 21%, 1Y return +14%. Large, stable sector with consistent demand.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Healthcare Service Providers (Hospitals, Diagnostics)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +23%, ROCE 25%, 1Y return +16%. Strong anchor.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Medical Equipment &amp; Supplies</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +26%, ROCE 15%. Emerging rocket within healthcare.</t>
+    </r>
+  </si>
+  <si>
+    <t>🟢 FMCG</t>
+  </si>
+  <si>
+    <r>
+      <t>Packaged Foods</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → ROCE 66%, sales growth +12%. Strong anchor with high margins.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Personal Care</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → ROCE 49%, steady demand, global FMCG anchor.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Edible Oil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +19%, ROCE 34%. Penny‑friendly FMCG anchor.</t>
+    </r>
+  </si>
+  <si>
+    <t>🚀 Aluminium / Zinc / Copper</t>
+  </si>
+  <si>
+    <r>
+      <t>Copper</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +62%, ROCE 41%, 1Y return +54%. Direct EV/renewables play.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Zinc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +39%, ROCE 69%, 1Y return +94%. Strongest rocket in metals.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Aluminium</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +19%, ROCE 19%, 1Y return +29%. Anchor in industrial metals.</t>
+    </r>
+  </si>
+  <si>
+    <t>⚡ Power</t>
+  </si>
+  <si>
+    <r>
+      <t>Power Distribution</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Sales growth +21%, ROCE 10%, 1Y return +45%. Utilities anchor.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Power Transmission</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → OPM 73%, ROCE 9%, 1Y return +4%. Stable margins.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Integrated Power Utilities</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → ROCE 15%, steady anchor with renewables + thermal mix.</t>
+    </r>
+  </si>
+  <si>
+    <t>🎯 Takeaway</t>
+  </si>
+  <si>
+    <r>
+      <t>Anchors (Stable)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Pharma, Healthcare Service Providers, Packaged Foods, Personal Care, Aluminium, Power Distribution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rockets (High Growth)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Copper, Zinc, Medical Equipment, Edible Oil.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Best balance: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>70% Anchors + 30% Rockets</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> across these four buckets.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6753,6 +7014,12 @@
         <fgColor rgb="FFBFE6FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -6766,7 +7033,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6781,8 +7048,13 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7122,9 +7394,122 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68095907-1B0A-4F3F-AFC8-1FCAE4547EF3}">
+  <dimension ref="A1:A21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="102.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
+        <v>2227</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="14" t="s">
+        <v>2229</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>2230</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="12" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>2232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="14" t="s">
+        <v>2233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="14" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="14" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="15" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M285"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7135,7 +7520,7 @@
     <col min="13" max="13" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7176,7 +7561,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -7217,7 +7602,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
@@ -7258,7 +7643,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>25</v>
       </c>
@@ -7299,7 +7684,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>25</v>
       </c>
@@ -7340,7 +7725,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>53</v>
       </c>
@@ -7381,7 +7766,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -7422,7 +7807,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>73</v>
       </c>
@@ -7463,7 +7848,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>73</v>
       </c>
@@ -7504,7 +7889,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>93</v>
       </c>
@@ -7545,7 +7930,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>104</v>
       </c>
@@ -7586,7 +7971,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>115</v>
       </c>
@@ -7627,7 +8012,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>126</v>
       </c>
@@ -7668,7 +8053,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>136</v>
       </c>
@@ -7709,7 +8094,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>147</v>
       </c>
@@ -7750,7 +8135,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>157</v>
       </c>
@@ -7791,7 +8176,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>162</v>
       </c>
@@ -7832,7 +8217,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>162</v>
       </c>
@@ -7873,7 +8258,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>182</v>
       </c>
@@ -7914,7 +8299,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>193</v>
       </c>
@@ -7955,7 +8340,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>200</v>
       </c>
@@ -7996,7 +8381,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>200</v>
       </c>
@@ -8037,7 +8422,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>219</v>
       </c>
@@ -8078,7 +8463,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>228</v>
       </c>
@@ -8119,7 +8504,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>228</v>
       </c>
@@ -8160,7 +8545,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>228</v>
       </c>
@@ -8201,7 +8586,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>228</v>
       </c>
@@ -8242,7 +8627,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>228</v>
       </c>
@@ -8283,7 +8668,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>228</v>
       </c>
@@ -8324,7 +8709,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>283</v>
       </c>
@@ -8365,7 +8750,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>292</v>
       </c>
@@ -8406,7 +8791,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>292</v>
       </c>
@@ -8447,7 +8832,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>292</v>
       </c>
@@ -8488,7 +8873,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>320</v>
       </c>
@@ -8529,7 +8914,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>320</v>
       </c>
@@ -8570,7 +8955,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>340</v>
       </c>
@@ -8611,7 +8996,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>340</v>
       </c>
@@ -8652,7 +9037,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>340</v>
       </c>
@@ -8693,7 +9078,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>340</v>
       </c>
@@ -8734,7 +9119,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
         <v>374</v>
       </c>
@@ -8775,7 +9160,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>374</v>
       </c>
@@ -8816,7 +9201,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>374</v>
       </c>
@@ -8857,7 +9242,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>398</v>
       </c>
@@ -8898,7 +9283,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>405</v>
       </c>
@@ -8939,7 +9324,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
         <v>405</v>
       </c>
@@ -8980,7 +9365,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
         <v>423</v>
       </c>
@@ -9021,7 +9406,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>434</v>
       </c>
@@ -9062,7 +9447,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>434</v>
       </c>
@@ -9103,7 +9488,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>448</v>
       </c>
@@ -9144,7 +9529,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>448</v>
       </c>
@@ -9185,7 +9570,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" s="10" t="s">
         <v>448</v>
       </c>
@@ -9226,7 +9611,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>473</v>
       </c>
@@ -9267,7 +9652,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>473</v>
       </c>
@@ -9308,7 +9693,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>473</v>
       </c>
@@ -9349,7 +9734,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
         <v>473</v>
       </c>
@@ -9390,7 +9775,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="10" t="s">
         <v>510</v>
       </c>
@@ -9431,7 +9816,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>520</v>
       </c>
@@ -9472,7 +9857,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>520</v>
       </c>
@@ -9513,7 +9898,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
         <v>520</v>
       </c>
@@ -9554,7 +9939,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
         <v>520</v>
       </c>
@@ -9595,7 +9980,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" s="10" t="s">
         <v>520</v>
       </c>
@@ -9636,7 +10021,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>561</v>
       </c>
@@ -9677,7 +10062,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>571</v>
       </c>
@@ -9718,7 +10103,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>582</v>
       </c>
@@ -9759,7 +10144,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" s="8" t="s">
         <v>582</v>
       </c>
@@ -9800,7 +10185,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
         <v>582</v>
       </c>
@@ -9841,7 +10226,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>608</v>
       </c>
@@ -9882,7 +10267,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>608</v>
       </c>
@@ -9923,7 +10308,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>626</v>
       </c>
@@ -9964,7 +10349,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" s="8" t="s">
         <v>626</v>
       </c>
@@ -10005,7 +10390,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
         <v>626</v>
       </c>
@@ -10046,7 +10431,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>626</v>
       </c>
@@ -10087,7 +10472,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>626</v>
       </c>
@@ -10128,7 +10513,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>626</v>
       </c>
@@ -10169,7 +10554,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" s="8" t="s">
         <v>626</v>
       </c>
@@ -10210,7 +10595,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
         <v>684</v>
       </c>
@@ -10251,7 +10636,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>684</v>
       </c>
@@ -10292,7 +10677,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>701</v>
       </c>
@@ -10333,7 +10718,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>701</v>
       </c>
@@ -10374,7 +10759,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" s="8" t="s">
         <v>701</v>
       </c>
@@ -10415,7 +10800,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" s="10" t="s">
         <v>724</v>
       </c>
@@ -10456,7 +10841,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>731</v>
       </c>
@@ -10497,7 +10882,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>731</v>
       </c>
@@ -10538,7 +10923,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>731</v>
       </c>
@@ -10579,7 +10964,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" s="8" t="s">
         <v>731</v>
       </c>
@@ -10620,7 +11005,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" s="10" t="s">
         <v>731</v>
       </c>
@@ -10661,7 +11046,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>731</v>
       </c>
@@ -10702,7 +11087,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>731</v>
       </c>
@@ -10743,7 +11128,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>790</v>
       </c>
@@ -10784,7 +11169,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" s="8" t="s">
         <v>797</v>
       </c>
@@ -10825,7 +11210,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" s="10" t="s">
         <v>797</v>
       </c>
@@ -10866,7 +11251,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>797</v>
       </c>
@@ -10907,7 +11292,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>822</v>
       </c>
@@ -10948,7 +11333,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>822</v>
       </c>
@@ -10989,7 +11374,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" s="8" t="s">
         <v>838</v>
       </c>
@@ -11030,7 +11415,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" s="10" t="s">
         <v>838</v>
       </c>
@@ -11071,7 +11456,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>854</v>
       </c>
@@ -11112,7 +11497,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>854</v>
       </c>
@@ -11153,7 +11538,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>854</v>
       </c>
@@ -11194,7 +11579,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" s="8" t="s">
         <v>854</v>
       </c>
@@ -11235,7 +11620,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" s="10" t="s">
         <v>854</v>
       </c>
@@ -11276,7 +11661,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>891</v>
       </c>
@@ -11317,7 +11702,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>891</v>
       </c>
@@ -11358,7 +11743,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" s="6" t="s">
         <v>891</v>
       </c>
@@ -11399,7 +11784,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" s="8" t="s">
         <v>891</v>
       </c>
@@ -11440,7 +11825,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" s="10" t="s">
         <v>891</v>
       </c>
@@ -11481,7 +11866,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>891</v>
       </c>
@@ -11522,7 +11907,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>891</v>
       </c>
@@ -11563,7 +11948,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" s="6" t="s">
         <v>891</v>
       </c>
@@ -11604,7 +11989,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" s="8" t="s">
         <v>891</v>
       </c>
@@ -11645,7 +12030,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" s="10" t="s">
         <v>891</v>
       </c>
@@ -11686,7 +12071,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>968</v>
       </c>
@@ -11727,7 +12112,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>977</v>
       </c>
@@ -11768,7 +12153,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" s="6" t="s">
         <v>984</v>
       </c>
@@ -11809,7 +12194,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" s="8" t="s">
         <v>991</v>
       </c>
@@ -11850,7 +12235,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A116" s="10" t="s">
         <v>1001</v>
       </c>
@@ -11891,7 +12276,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>1010</v>
       </c>
@@ -11932,7 +12317,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>1020</v>
       </c>
@@ -11973,7 +12358,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A119" s="6" t="s">
         <v>1020</v>
       </c>
@@ -12014,7 +12399,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A120" s="8" t="s">
         <v>1037</v>
       </c>
@@ -12055,7 +12440,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A121" s="10" t="s">
         <v>1046</v>
       </c>
@@ -12096,7 +12481,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>1054</v>
       </c>
@@ -12137,7 +12522,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A123" s="4" t="s">
         <v>1062</v>
       </c>
@@ -12178,7 +12563,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A124" s="6" t="s">
         <v>1062</v>
       </c>
@@ -12219,7 +12604,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A125" s="8" t="s">
         <v>1062</v>
       </c>
@@ -12260,7 +12645,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A126" s="10" t="s">
         <v>1062</v>
       </c>
@@ -12301,7 +12686,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>1062</v>
       </c>
@@ -12342,7 +12727,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
         <v>1062</v>
       </c>
@@ -12383,7 +12768,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>1110</v>
       </c>
@@ -12424,7 +12809,7 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A130" s="8" t="s">
         <v>1118</v>
       </c>
@@ -12465,7 +12850,7 @@
         <v>1126</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A131" s="10" t="s">
         <v>1118</v>
       </c>
@@ -12506,7 +12891,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>1118</v>
       </c>
@@ -12547,7 +12932,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A133" s="4" t="s">
         <v>1118</v>
       </c>
@@ -12588,7 +12973,7 @@
         <v>1146</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A134" s="6" t="s">
         <v>1118</v>
       </c>
@@ -12629,7 +13014,7 @@
         <v>1151</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A135" s="8" t="s">
         <v>1118</v>
       </c>
@@ -12670,7 +13055,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A136" s="10" t="s">
         <v>1118</v>
       </c>
@@ -12711,7 +13096,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>1166</v>
       </c>
@@ -12752,7 +13137,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
         <v>1166</v>
       </c>
@@ -12793,7 +13178,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
         <v>1166</v>
       </c>
@@ -12834,7 +13219,7 @@
         <v>1191</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A140" s="8" t="s">
         <v>1166</v>
       </c>
@@ -12875,7 +13260,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A141" s="10" t="s">
         <v>1166</v>
       </c>
@@ -12916,7 +13301,7 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>1166</v>
       </c>
@@ -12957,7 +13342,7 @@
         <v>1215</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A143" s="4" t="s">
         <v>1166</v>
       </c>
@@ -12998,7 +13383,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A144" s="6" t="s">
         <v>1166</v>
       </c>
@@ -13039,7 +13424,7 @@
         <v>1232</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A145" s="8" t="s">
         <v>1166</v>
       </c>
@@ -13080,7 +13465,7 @@
         <v>1242</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A146" s="10" t="s">
         <v>1243</v>
       </c>
@@ -13121,7 +13506,7 @@
         <v>1248</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>1243</v>
       </c>
@@ -13162,7 +13547,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A148" s="4" t="s">
         <v>1243</v>
       </c>
@@ -13203,7 +13588,7 @@
         <v>1262</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A149" s="6" t="s">
         <v>1243</v>
       </c>
@@ -13244,7 +13629,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A150" s="8" t="s">
         <v>1268</v>
       </c>
@@ -13285,7 +13670,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A151" s="10" t="s">
         <v>1268</v>
       </c>
@@ -13326,7 +13711,7 @@
         <v>1282</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>1283</v>
       </c>
@@ -13367,7 +13752,7 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
         <v>1292</v>
       </c>
@@ -13408,7 +13793,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A154" s="6" t="s">
         <v>1292</v>
       </c>
@@ -13449,7 +13834,7 @@
         <v>1306</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A155" s="8" t="s">
         <v>1292</v>
       </c>
@@ -13490,7 +13875,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A156" s="10" t="s">
         <v>1292</v>
       </c>
@@ -13531,7 +13916,7 @@
         <v>1320</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>1292</v>
       </c>
@@ -13572,7 +13957,7 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
         <v>1292</v>
       </c>
@@ -13613,7 +13998,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A159" s="6" t="s">
         <v>1292</v>
       </c>
@@ -13654,7 +14039,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A160" s="8" t="s">
         <v>1292</v>
       </c>
@@ -13695,7 +14080,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A161" s="10" t="s">
         <v>1351</v>
       </c>
@@ -13736,7 +14121,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>1351</v>
       </c>
@@ -13777,7 +14162,7 @@
         <v>1366</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
         <v>1351</v>
       </c>
@@ -13818,7 +14203,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A164" s="6" t="s">
         <v>1351</v>
       </c>
@@ -13859,7 +14244,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A165" s="8" t="s">
         <v>1351</v>
       </c>
@@ -13900,7 +14285,7 @@
         <v>1389</v>
       </c>
     </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A166" s="10" t="s">
         <v>1351</v>
       </c>
@@ -13941,7 +14326,7 @@
         <v>1397</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>1351</v>
       </c>
@@ -13982,7 +14367,7 @@
         <v>1406</v>
       </c>
     </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A168" s="4" t="s">
         <v>1351</v>
       </c>
@@ -14023,7 +14408,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A169" s="6" t="s">
         <v>1351</v>
       </c>
@@ -14064,7 +14449,7 @@
         <v>1419</v>
       </c>
     </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A170" s="8" t="s">
         <v>1420</v>
       </c>
@@ -14105,7 +14490,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A171" s="10" t="s">
         <v>1430</v>
       </c>
@@ -14146,7 +14531,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>1430</v>
       </c>
@@ -14187,7 +14572,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A173" s="4" t="s">
         <v>1430</v>
       </c>
@@ -14228,7 +14613,7 @@
         <v>1454</v>
       </c>
     </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A174" s="6" t="s">
         <v>1455</v>
       </c>
@@ -14269,7 +14654,7 @@
         <v>1461</v>
       </c>
     </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A175" s="8" t="s">
         <v>1462</v>
       </c>
@@ -14310,7 +14695,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A176" s="10" t="s">
         <v>1471</v>
       </c>
@@ -14351,7 +14736,7 @@
         <v>1478</v>
       </c>
     </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>1471</v>
       </c>
@@ -14392,7 +14777,7 @@
         <v>1482</v>
       </c>
     </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A178" s="4" t="s">
         <v>1471</v>
       </c>
@@ -14433,7 +14818,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>1471</v>
       </c>
@@ -14474,7 +14859,7 @@
         <v>1497</v>
       </c>
     </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A180" s="8" t="s">
         <v>1471</v>
       </c>
@@ -14515,7 +14900,7 @@
         <v>1503</v>
       </c>
     </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A181" s="10" t="s">
         <v>1504</v>
       </c>
@@ -14556,7 +14941,7 @@
         <v>1512</v>
       </c>
     </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>1504</v>
       </c>
@@ -14597,7 +14982,7 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A183" s="4" t="s">
         <v>1504</v>
       </c>
@@ -14638,7 +15023,7 @@
         <v>1523</v>
       </c>
     </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A184" s="6" t="s">
         <v>1504</v>
       </c>
@@ -14679,7 +15064,7 @@
         <v>1529</v>
       </c>
     </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A185" s="8" t="s">
         <v>1504</v>
       </c>
@@ -14720,7 +15105,7 @@
         <v>1535</v>
       </c>
     </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A186" s="10" t="s">
         <v>1536</v>
       </c>
@@ -14761,7 +15146,7 @@
         <v>1544</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>1545</v>
       </c>
@@ -14802,7 +15187,7 @@
         <v>1551</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A188" s="4" t="s">
         <v>1552</v>
       </c>
@@ -14843,7 +15228,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A189" s="6" t="s">
         <v>1552</v>
       </c>
@@ -14884,7 +15269,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A190" s="8" t="s">
         <v>1552</v>
       </c>
@@ -14925,7 +15310,7 @@
         <v>1574</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A191" s="10" t="s">
         <v>1552</v>
       </c>
@@ -14966,7 +15351,7 @@
         <v>1580</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>1552</v>
       </c>
@@ -15007,7 +15392,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A193" s="4" t="s">
         <v>1552</v>
       </c>
@@ -15048,7 +15433,7 @@
         <v>1595</v>
       </c>
     </row>
-    <row r="194" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A194" s="6" t="s">
         <v>1552</v>
       </c>
@@ -15089,7 +15474,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="195" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A195" s="8" t="s">
         <v>1552</v>
       </c>
@@ -15130,7 +15515,7 @@
         <v>1608</v>
       </c>
     </row>
-    <row r="196" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A196" s="10" t="s">
         <v>1552</v>
       </c>
@@ -15171,7 +15556,7 @@
         <v>1614</v>
       </c>
     </row>
-    <row r="197" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>1552</v>
       </c>
@@ -15212,7 +15597,7 @@
         <v>1621</v>
       </c>
     </row>
-    <row r="198" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A198" s="4" t="s">
         <v>1622</v>
       </c>
@@ -15253,7 +15638,7 @@
         <v>1630</v>
       </c>
     </row>
-    <row r="199" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A199" s="6" t="s">
         <v>1622</v>
       </c>
@@ -15294,7 +15679,7 @@
         <v>1639</v>
       </c>
     </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A200" s="8" t="s">
         <v>1622</v>
       </c>
@@ -15335,7 +15720,7 @@
         <v>1644</v>
       </c>
     </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A201" s="10" t="s">
         <v>1622</v>
       </c>
@@ -15376,7 +15761,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>1622</v>
       </c>
@@ -15417,7 +15802,7 @@
         <v>1657</v>
       </c>
     </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A203" s="4" t="s">
         <v>1622</v>
       </c>
@@ -15458,7 +15843,7 @@
         <v>1665</v>
       </c>
     </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A204" s="6" t="s">
         <v>1666</v>
       </c>
@@ -15499,7 +15884,7 @@
         <v>1671</v>
       </c>
     </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A205" s="8" t="s">
         <v>1666</v>
       </c>
@@ -15540,7 +15925,7 @@
         <v>1678</v>
       </c>
     </row>
-    <row r="206" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A206" s="10" t="s">
         <v>1679</v>
       </c>
@@ -15581,7 +15966,7 @@
         <v>1684</v>
       </c>
     </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>1685</v>
       </c>
@@ -15622,7 +16007,7 @@
         <v>1690</v>
       </c>
     </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A208" s="4" t="s">
         <v>1691</v>
       </c>
@@ -15663,7 +16048,7 @@
         <v>1698</v>
       </c>
     </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A209" s="6" t="s">
         <v>1699</v>
       </c>
@@ -15704,7 +16089,7 @@
         <v>1706</v>
       </c>
     </row>
-    <row r="210" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A210" s="8" t="s">
         <v>1699</v>
       </c>
@@ -15745,7 +16130,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="211" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A211" s="10" t="s">
         <v>1712</v>
       </c>
@@ -15786,7 +16171,7 @@
         <v>1718</v>
       </c>
     </row>
-    <row r="212" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>1712</v>
       </c>
@@ -15827,7 +16212,7 @@
         <v>1724</v>
       </c>
     </row>
-    <row r="213" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A213" s="4" t="s">
         <v>1712</v>
       </c>
@@ -15868,7 +16253,7 @@
         <v>1730</v>
       </c>
     </row>
-    <row r="214" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A214" s="6" t="s">
         <v>1731</v>
       </c>
@@ -15909,7 +16294,7 @@
         <v>1738</v>
       </c>
     </row>
-    <row r="215" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A215" s="8" t="s">
         <v>1731</v>
       </c>
@@ -15950,7 +16335,7 @@
         <v>1744</v>
       </c>
     </row>
-    <row r="216" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A216" s="10" t="s">
         <v>1745</v>
       </c>
@@ -15991,7 +16376,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>1745</v>
       </c>
@@ -16032,7 +16417,7 @@
         <v>1758</v>
       </c>
     </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A218" s="4" t="s">
         <v>1759</v>
       </c>
@@ -16073,7 +16458,7 @@
         <v>1766</v>
       </c>
     </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A219" s="6" t="s">
         <v>1759</v>
       </c>
@@ -16114,7 +16499,7 @@
         <v>1775</v>
       </c>
     </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A220" s="8" t="s">
         <v>1759</v>
       </c>
@@ -16155,7 +16540,7 @@
         <v>1781</v>
       </c>
     </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A221" s="10" t="s">
         <v>1759</v>
       </c>
@@ -16196,7 +16581,7 @@
         <v>1788</v>
       </c>
     </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>1789</v>
       </c>
@@ -16237,7 +16622,7 @@
         <v>1796</v>
       </c>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A223" s="4" t="s">
         <v>1797</v>
       </c>
@@ -16278,7 +16663,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A224" s="6" t="s">
         <v>1797</v>
       </c>
@@ -16319,7 +16704,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="225" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A225" s="8" t="s">
         <v>1810</v>
       </c>
@@ -16360,7 +16745,7 @@
         <v>1815</v>
       </c>
     </row>
-    <row r="226" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A226" s="10" t="s">
         <v>1816</v>
       </c>
@@ -16401,7 +16786,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="227" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
         <v>1824</v>
       </c>
@@ -16442,7 +16827,7 @@
         <v>1832</v>
       </c>
     </row>
-    <row r="228" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A228" s="4" t="s">
         <v>1824</v>
       </c>
@@ -16483,7 +16868,7 @@
         <v>1839</v>
       </c>
     </row>
-    <row r="229" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A229" s="6" t="s">
         <v>1840</v>
       </c>
@@ -16524,7 +16909,7 @@
         <v>1846</v>
       </c>
     </row>
-    <row r="230" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A230" s="8" t="s">
         <v>1840</v>
       </c>
@@ -16565,7 +16950,7 @@
         <v>1853</v>
       </c>
     </row>
-    <row r="231" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A231" s="10" t="s">
         <v>1840</v>
       </c>
@@ -16606,7 +16991,7 @@
         <v>1860</v>
       </c>
     </row>
-    <row r="232" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
         <v>1840</v>
       </c>
@@ -16647,7 +17032,7 @@
         <v>1866</v>
       </c>
     </row>
-    <row r="233" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A233" s="4" t="s">
         <v>1840</v>
       </c>
@@ -16688,7 +17073,7 @@
         <v>1874</v>
       </c>
     </row>
-    <row r="234" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A234" s="6" t="s">
         <v>1875</v>
       </c>
@@ -16729,7 +17114,7 @@
         <v>1882</v>
       </c>
     </row>
-    <row r="235" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A235" s="8" t="s">
         <v>1875</v>
       </c>
@@ -16770,7 +17155,7 @@
         <v>1888</v>
       </c>
     </row>
-    <row r="236" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A236" s="10" t="s">
         <v>1875</v>
       </c>
@@ -16811,7 +17196,7 @@
         <v>1896</v>
       </c>
     </row>
-    <row r="237" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A237" s="2" t="s">
         <v>1897</v>
       </c>
@@ -16852,7 +17237,7 @@
         <v>1904</v>
       </c>
     </row>
-    <row r="238" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A238" s="4" t="s">
         <v>1905</v>
       </c>
@@ -16893,7 +17278,7 @@
         <v>1912</v>
       </c>
     </row>
-    <row r="239" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A239" s="6" t="s">
         <v>1905</v>
       </c>
@@ -16934,7 +17319,7 @@
         <v>1917</v>
       </c>
     </row>
-    <row r="240" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A240" s="8" t="s">
         <v>1918</v>
       </c>
@@ -16975,7 +17360,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="241" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A241" s="10" t="s">
         <v>1918</v>
       </c>
@@ -17016,7 +17401,7 @@
         <v>1928</v>
       </c>
     </row>
-    <row r="242" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A242" s="2" t="s">
         <v>1929</v>
       </c>
@@ -17057,7 +17442,7 @@
         <v>1934</v>
       </c>
     </row>
-    <row r="243" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A243" s="4" t="s">
         <v>1935</v>
       </c>
@@ -17098,7 +17483,7 @@
         <v>1943</v>
       </c>
     </row>
-    <row r="244" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A244" s="6" t="s">
         <v>1935</v>
       </c>
@@ -17139,7 +17524,7 @@
         <v>1951</v>
       </c>
     </row>
-    <row r="245" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A245" s="8" t="s">
         <v>1935</v>
       </c>
@@ -17180,7 +17565,7 @@
         <v>1956</v>
       </c>
     </row>
-    <row r="246" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A246" s="10" t="s">
         <v>1957</v>
       </c>
@@ -17221,7 +17606,7 @@
         <v>1965</v>
       </c>
     </row>
-    <row r="247" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A247" s="2" t="s">
         <v>1957</v>
       </c>
@@ -17262,7 +17647,7 @@
         <v>1971</v>
       </c>
     </row>
-    <row r="248" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A248" s="4" t="s">
         <v>1972</v>
       </c>
@@ -17303,7 +17688,7 @@
         <v>1979</v>
       </c>
     </row>
-    <row r="249" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A249" s="6" t="s">
         <v>1972</v>
       </c>
@@ -17344,7 +17729,7 @@
         <v>1986</v>
       </c>
     </row>
-    <row r="250" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A250" s="8" t="s">
         <v>1972</v>
       </c>
@@ -17385,7 +17770,7 @@
         <v>1992</v>
       </c>
     </row>
-    <row r="251" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A251" s="10" t="s">
         <v>1972</v>
       </c>
@@ -17426,7 +17811,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="252" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A252" s="2" t="s">
         <v>1972</v>
       </c>
@@ -17467,7 +17852,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="253" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A253" s="4" t="s">
         <v>2009</v>
       </c>
@@ -17508,7 +17893,7 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="254" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A254" s="6" t="s">
         <v>2009</v>
       </c>
@@ -17549,7 +17934,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="255" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A255" s="8" t="s">
         <v>2027</v>
       </c>
@@ -17590,7 +17975,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="256" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A256" s="10" t="s">
         <v>2027</v>
       </c>
@@ -17631,7 +18016,7 @@
         <v>2036</v>
       </c>
     </row>
-    <row r="257" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A257" s="2" t="s">
         <v>2027</v>
       </c>
@@ -17672,7 +18057,7 @@
         <v>2042</v>
       </c>
     </row>
-    <row r="258" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A258" s="4" t="s">
         <v>2043</v>
       </c>
@@ -17713,7 +18098,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="259" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A259" s="6" t="s">
         <v>2049</v>
       </c>
@@ -17754,7 +18139,7 @@
         <v>2057</v>
       </c>
     </row>
-    <row r="260" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A260" s="8" t="s">
         <v>2049</v>
       </c>
@@ -17795,7 +18180,7 @@
         <v>2061</v>
       </c>
     </row>
-    <row r="261" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A261" s="10" t="s">
         <v>2049</v>
       </c>
@@ -17836,7 +18221,7 @@
         <v>2069</v>
       </c>
     </row>
-    <row r="262" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A262" s="2" t="s">
         <v>2070</v>
       </c>
@@ -17877,7 +18262,7 @@
         <v>2076</v>
       </c>
     </row>
-    <row r="263" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A263" s="4" t="s">
         <v>2070</v>
       </c>
@@ -17918,7 +18303,7 @@
         <v>2081</v>
       </c>
     </row>
-    <row r="264" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A264" s="6" t="s">
         <v>2070</v>
       </c>
@@ -17959,7 +18344,7 @@
         <v>2087</v>
       </c>
     </row>
-    <row r="265" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A265" s="8" t="s">
         <v>2070</v>
       </c>
@@ -18000,7 +18385,7 @@
         <v>2095</v>
       </c>
     </row>
-    <row r="266" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A266" s="10" t="s">
         <v>2096</v>
       </c>
@@ -18041,7 +18426,7 @@
         <v>2102</v>
       </c>
     </row>
-    <row r="267" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A267" s="2" t="s">
         <v>2103</v>
       </c>
@@ -18082,7 +18467,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="268" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A268" s="4" t="s">
         <v>2103</v>
       </c>
@@ -18123,7 +18508,7 @@
         <v>2119</v>
       </c>
     </row>
-    <row r="269" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A269" s="6" t="s">
         <v>2120</v>
       </c>
@@ -18164,7 +18549,7 @@
         <v>2126</v>
       </c>
     </row>
-    <row r="270" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A270" s="8" t="s">
         <v>2120</v>
       </c>
@@ -18205,7 +18590,7 @@
         <v>2132</v>
       </c>
     </row>
-    <row r="271" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A271" s="10" t="s">
         <v>2120</v>
       </c>
@@ -18246,7 +18631,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="272" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A272" s="2" t="s">
         <v>2120</v>
       </c>
@@ -18287,7 +18672,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="273" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A273" s="4" t="s">
         <v>2120</v>
       </c>
@@ -18328,7 +18713,7 @@
         <v>2156</v>
       </c>
     </row>
-    <row r="274" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A274" s="6" t="s">
         <v>2120</v>
       </c>
@@ -18369,7 +18754,7 @@
         <v>2163</v>
       </c>
     </row>
-    <row r="275" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A275" s="8" t="s">
         <v>2164</v>
       </c>
@@ -18410,7 +18795,7 @@
         <v>2170</v>
       </c>
     </row>
-    <row r="276" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A276" s="10" t="s">
         <v>2164</v>
       </c>
@@ -18451,7 +18836,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="277" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A277" s="2" t="s">
         <v>2164</v>
       </c>
@@ -18492,7 +18877,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="278" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A278" s="4" t="s">
         <v>2164</v>
       </c>
@@ -18533,7 +18918,7 @@
         <v>2188</v>
       </c>
     </row>
-    <row r="279" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A279" s="6" t="s">
         <v>2164</v>
       </c>
@@ -18574,7 +18959,7 @@
         <v>2192</v>
       </c>
     </row>
-    <row r="280" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A280" s="8" t="s">
         <v>2164</v>
       </c>
@@ -18615,7 +19000,7 @@
         <v>2198</v>
       </c>
     </row>
-    <row r="281" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A281" s="10" t="s">
         <v>2164</v>
       </c>
@@ -18656,7 +19041,7 @@
         <v>2203</v>
       </c>
     </row>
-    <row r="282" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A282" s="2" t="s">
         <v>2164</v>
       </c>
@@ -18697,7 +19082,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="283" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A283" s="4" t="s">
         <v>2164</v>
       </c>
@@ -18738,7 +19123,7 @@
         <v>2215</v>
       </c>
     </row>
-    <row r="284" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A284" s="6" t="s">
         <v>2164</v>
       </c>
@@ -18779,7 +19164,7 @@
         <v>2219</v>
       </c>
     </row>
-    <row r="285" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A285" s="8" t="s">
         <v>2220</v>
       </c>
@@ -18821,660 +19206,578 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
+  <autoFilter ref="A1:M1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" tooltip="https://www.screener.in/company/WARDINMOBI/"/>
-    <hyperlink ref="M2" r:id="rId2" tooltip="https://www.screener.in/company/WARDINMOBI/"/>
-    <hyperlink ref="B3" r:id="rId3" tooltip="https://www.screener.in/company/539310/"/>
-    <hyperlink ref="M3" r:id="rId4" tooltip="https://www.screener.in/company/539310/"/>
-    <hyperlink ref="B4" r:id="rId5" tooltip="https://www.screener.in/company/543341/consolidated/"/>
-    <hyperlink ref="M4" r:id="rId6" tooltip="https://www.screener.in/company/543341/consolidated/"/>
-    <hyperlink ref="B5" r:id="rId7" tooltip="https://www.screener.in/company/526441/consolidated/"/>
-    <hyperlink ref="M5" r:id="rId8" tooltip="https://www.screener.in/company/526441/consolidated/"/>
-    <hyperlink ref="B6" r:id="rId9" tooltip="https://www.screener.in/company/SPICEJET/"/>
-    <hyperlink ref="M6" r:id="rId10" tooltip="https://www.screener.in/company/SPICEJET/"/>
-    <hyperlink ref="B7" r:id="rId11" tooltip="https://www.screener.in/company/531869/"/>
-    <hyperlink ref="M7" r:id="rId12" tooltip="https://www.screener.in/company/531869/"/>
-    <hyperlink ref="B8" r:id="rId13" tooltip="https://www.screener.in/company/513502/"/>
-    <hyperlink ref="M8" r:id="rId14" tooltip="https://www.screener.in/company/513502/"/>
-    <hyperlink ref="B9" r:id="rId15" tooltip="https://www.screener.in/company/RAJMET/"/>
-    <hyperlink ref="M9" r:id="rId16" tooltip="https://www.screener.in/company/RAJMET/"/>
-    <hyperlink ref="B10" r:id="rId17" tooltip="https://www.screener.in/company/538731/"/>
-    <hyperlink ref="M10" r:id="rId18" tooltip="https://www.screener.in/company/538731/"/>
-    <hyperlink ref="B11" r:id="rId19" tooltip="https://www.screener.in/company/AJOONI/"/>
-    <hyperlink ref="M11" r:id="rId20" tooltip="https://www.screener.in/company/AJOONI/"/>
-    <hyperlink ref="B12" r:id="rId21" tooltip="https://www.screener.in/company/IVC/consolidated/"/>
-    <hyperlink ref="M12" r:id="rId22" tooltip="https://www.screener.in/company/IVC/consolidated/"/>
-    <hyperlink ref="B13" r:id="rId23" tooltip="https://www.screener.in/company/539402/"/>
-    <hyperlink ref="M13" r:id="rId24" tooltip="https://www.screener.in/company/539402/"/>
-    <hyperlink ref="B14" r:id="rId25" tooltip="https://www.screener.in/company/539470/"/>
-    <hyperlink ref="M14" r:id="rId26" tooltip="https://www.screener.in/company/539470/"/>
-    <hyperlink ref="B15" r:id="rId27" tooltip="https://www.screener.in/company/COMFINTE/consolidated/"/>
-    <hyperlink ref="M15" r:id="rId28" tooltip="https://www.screener.in/company/COMFINTE/consolidated/"/>
-    <hyperlink ref="B16" r:id="rId29" tooltip="https://www.screener.in/company/532139/"/>
-    <hyperlink ref="M16" r:id="rId30" tooltip="https://www.screener.in/company/532139/"/>
-    <hyperlink ref="B17" r:id="rId31" tooltip="https://www.screener.in/company/538706/"/>
-    <hyperlink ref="M17" r:id="rId32" tooltip="https://www.screener.in/company/538706/"/>
-    <hyperlink ref="B18" r:id="rId33" tooltip="https://www.screener.in/company/BCP/"/>
-    <hyperlink ref="M18" r:id="rId34" tooltip="https://www.screener.in/company/BCP/"/>
-    <hyperlink ref="B19" r:id="rId35" tooltip="https://www.screener.in/company/513418/"/>
-    <hyperlink ref="M19" r:id="rId36" tooltip="https://www.screener.in/company/513418/"/>
-    <hyperlink ref="B20" r:id="rId37" tooltip="https://www.screener.in/company/526941/"/>
-    <hyperlink ref="M20" r:id="rId38" tooltip="https://www.screener.in/company/526941/"/>
-    <hyperlink ref="B21" r:id="rId39" tooltip="https://www.screener.in/company/EXXARO/consolidated/"/>
-    <hyperlink ref="M21" r:id="rId40" tooltip="https://www.screener.in/company/EXXARO/consolidated/"/>
-    <hyperlink ref="B22" r:id="rId41" tooltip="https://www.screener.in/company/515085/"/>
-    <hyperlink ref="M22" r:id="rId42" tooltip="https://www.screener.in/company/515085/"/>
-    <hyperlink ref="B23" r:id="rId43" tooltip="https://www.screener.in/company/ELITECON/consolidated/"/>
-    <hyperlink ref="M23" r:id="rId44" tooltip="https://www.screener.in/company/ELITECON/consolidated/"/>
-    <hyperlink ref="B24" r:id="rId45" tooltip="https://www.screener.in/company/SEPC/consolidated/"/>
-    <hyperlink ref="M24" r:id="rId46" tooltip="https://www.screener.in/company/SEPC/consolidated/"/>
-    <hyperlink ref="B25" r:id="rId47" tooltip="https://www.screener.in/company/DBEIL/"/>
-    <hyperlink ref="M25" r:id="rId48" tooltip="https://www.screener.in/company/DBEIL/"/>
-    <hyperlink ref="B26" r:id="rId49" tooltip="https://www.screener.in/company/MADHAVIPL/consolidated/"/>
-    <hyperlink ref="M26" r:id="rId50" tooltip="https://www.screener.in/company/MADHAVIPL/consolidated/"/>
-    <hyperlink ref="B27" r:id="rId51" tooltip="https://www.screener.in/company/TICL/consolidated/"/>
-    <hyperlink ref="M27" r:id="rId52" tooltip="https://www.screener.in/company/TICL/consolidated/"/>
-    <hyperlink ref="B28" r:id="rId53" tooltip="https://www.screener.in/company/SADBHAV/consolidated/"/>
-    <hyperlink ref="M28" r:id="rId54" tooltip="https://www.screener.in/company/SADBHAV/consolidated/"/>
-    <hyperlink ref="B29" r:id="rId55" tooltip="https://www.screener.in/company/NAVKARURB/"/>
-    <hyperlink ref="M29" r:id="rId56" tooltip="https://www.screener.in/company/NAVKARURB/"/>
-    <hyperlink ref="B30" r:id="rId57" tooltip="https://www.screener.in/company/513579/"/>
-    <hyperlink ref="M30" r:id="rId58" tooltip="https://www.screener.in/company/513579/"/>
-    <hyperlink ref="B31" r:id="rId59" tooltip="https://www.screener.in/company/SADHNANIQ/consolidated/"/>
-    <hyperlink ref="M31" r:id="rId60" tooltip="https://www.screener.in/company/SADHNANIQ/consolidated/"/>
-    <hyperlink ref="B32" r:id="rId61" tooltip="https://www.screener.in/company/514440/"/>
-    <hyperlink ref="M32" r:id="rId62" tooltip="https://www.screener.in/company/514440/"/>
-    <hyperlink ref="B33" r:id="rId63" tooltip="https://www.screener.in/company/524564/"/>
-    <hyperlink ref="M33" r:id="rId64" tooltip="https://www.screener.in/company/524564/"/>
-    <hyperlink ref="B34" r:id="rId65" tooltip="https://www.screener.in/company/EMPOWER/consolidated/"/>
-    <hyperlink ref="M34" r:id="rId66" tooltip="https://www.screener.in/company/EMPOWER/consolidated/"/>
-    <hyperlink ref="B35" r:id="rId67" tooltip="https://www.screener.in/company/GVPTECH/"/>
-    <hyperlink ref="M35" r:id="rId68" tooltip="https://www.screener.in/company/GVPTECH/"/>
-    <hyperlink ref="B36" r:id="rId69" tooltip="https://www.screener.in/company/517393/"/>
-    <hyperlink ref="M36" r:id="rId70" tooltip="https://www.screener.in/company/517393/"/>
-    <hyperlink ref="B37" r:id="rId71" tooltip="https://www.screener.in/company/CEREBRAINT/consolidated/"/>
-    <hyperlink ref="M37" r:id="rId72" tooltip="https://www.screener.in/company/CEREBRAINT/consolidated/"/>
-    <hyperlink ref="B38" r:id="rId73" tooltip="https://www.screener.in/company/517356/"/>
-    <hyperlink ref="M38" r:id="rId74" tooltip="https://www.screener.in/company/517356/"/>
-    <hyperlink ref="B39" r:id="rId75" tooltip="https://www.screener.in/company/512175/"/>
-    <hyperlink ref="M39" r:id="rId76" tooltip="https://www.screener.in/company/512175/"/>
-    <hyperlink ref="B40" r:id="rId77" tooltip="https://www.screener.in/company/511716/"/>
-    <hyperlink ref="M40" r:id="rId78" tooltip="https://www.screener.in/company/511716/"/>
-    <hyperlink ref="B41" r:id="rId79" tooltip="https://www.screener.in/company/539149/consolidated/"/>
-    <hyperlink ref="M41" r:id="rId80" tooltip="https://www.screener.in/company/539149/consolidated/"/>
-    <hyperlink ref="B42" r:id="rId81" tooltip="https://www.screener.in/company/503641/consolidated/"/>
-    <hyperlink ref="M42" r:id="rId82" tooltip="https://www.screener.in/company/503641/consolidated/"/>
-    <hyperlink ref="B43" r:id="rId83" tooltip="https://www.screener.in/company/517399/"/>
-    <hyperlink ref="M43" r:id="rId84" tooltip="https://www.screener.in/company/517399/"/>
-    <hyperlink ref="B44" r:id="rId85" tooltip="https://www.screener.in/company/543546/consolidated/"/>
-    <hyperlink ref="M44" r:id="rId86" tooltip="https://www.screener.in/company/543546/consolidated/"/>
-    <hyperlink ref="B45" r:id="rId87" tooltip="https://www.screener.in/company/540955/"/>
-    <hyperlink ref="M45" r:id="rId88" tooltip="https://www.screener.in/company/540955/"/>
-    <hyperlink ref="B46" r:id="rId89" tooltip="https://www.screener.in/company/BTML/consolidated/"/>
-    <hyperlink ref="M46" r:id="rId90" tooltip="https://www.screener.in/company/BTML/consolidated/"/>
-    <hyperlink ref="B47" r:id="rId91" tooltip="https://www.screener.in/company/539519/consolidated/"/>
-    <hyperlink ref="M47" r:id="rId92" tooltip="https://www.screener.in/company/539519/consolidated/"/>
-    <hyperlink ref="B48" r:id="rId93" tooltip="https://www.screener.in/company/539673/"/>
-    <hyperlink ref="M48" r:id="rId94" tooltip="https://www.screener.in/company/539673/"/>
-    <hyperlink ref="B49" r:id="rId95" tooltip="https://www.screener.in/company/542802/consolidated/"/>
-    <hyperlink ref="M49" r:id="rId96" tooltip="https://www.screener.in/company/542802/consolidated/"/>
-    <hyperlink ref="B50" r:id="rId97" tooltip="https://www.screener.in/company/512257/"/>
-    <hyperlink ref="M50" r:id="rId98" tooltip="https://www.screener.in/company/512257/"/>
-    <hyperlink ref="B51" r:id="rId99" tooltip="https://www.screener.in/company/511463/"/>
-    <hyperlink ref="M51" r:id="rId100" tooltip="https://www.screener.in/company/511463/"/>
-    <hyperlink ref="B52" r:id="rId101" tooltip="https://www.screener.in/company/526935/"/>
-    <hyperlink ref="M52" r:id="rId102" tooltip="https://www.screener.in/company/526935/"/>
-    <hyperlink ref="B53" r:id="rId103" tooltip="https://www.screener.in/company/ALANKIT/consolidated/"/>
-    <hyperlink ref="M53" r:id="rId104" tooltip="https://www.screener.in/company/ALANKIT/consolidated/"/>
-    <hyperlink ref="B54" r:id="rId105" tooltip="https://www.screener.in/company/511557/"/>
-    <hyperlink ref="M54" r:id="rId106" tooltip="https://www.screener.in/company/511557/"/>
-    <hyperlink ref="B55" r:id="rId107" tooltip="https://www.screener.in/company/RUCHINFRA/consolidated/"/>
-    <hyperlink ref="M55" r:id="rId108" tooltip="https://www.screener.in/company/RUCHINFRA/consolidated/"/>
-    <hyperlink ref="B56" r:id="rId109" tooltip="https://www.screener.in/company/DAVANGERE/"/>
-    <hyperlink ref="M56" r:id="rId110" tooltip="https://www.screener.in/company/DAVANGERE/"/>
-    <hyperlink ref="B57" r:id="rId111" tooltip="https://www.screener.in/company/OSIAHYPER/"/>
-    <hyperlink ref="M57" r:id="rId112" tooltip="https://www.screener.in/company/OSIAHYPER/"/>
-    <hyperlink ref="B58" r:id="rId113" tooltip="https://www.screener.in/company/FLFL/consolidated/"/>
-    <hyperlink ref="M58" r:id="rId114" tooltip="https://www.screener.in/company/FLFL/consolidated/"/>
-    <hyperlink ref="B59" r:id="rId115" tooltip="https://www.screener.in/company/FEL/"/>
-    <hyperlink ref="M59" r:id="rId116" tooltip="https://www.screener.in/company/FEL/"/>
-    <hyperlink ref="B60" r:id="rId117" tooltip="https://www.screener.in/company/534708/"/>
-    <hyperlink ref="M60" r:id="rId118" tooltip="https://www.screener.in/company/534708/"/>
-    <hyperlink ref="B61" r:id="rId119" tooltip="https://www.screener.in/company/FELDVR/"/>
-    <hyperlink ref="M61" r:id="rId120" tooltip="https://www.screener.in/company/FELDVR/"/>
-    <hyperlink ref="B62" r:id="rId121" tooltip="https://www.screener.in/company/YCCL/consolidated/"/>
-    <hyperlink ref="M62" r:id="rId122" tooltip="https://www.screener.in/company/YCCL/consolidated/"/>
-    <hyperlink ref="B63" r:id="rId123" tooltip="https://www.screener.in/company/UMESLTD/consolidated/"/>
-    <hyperlink ref="M63" r:id="rId124" tooltip="https://www.screener.in/company/UMESLTD/consolidated/"/>
-    <hyperlink ref="B64" r:id="rId125" tooltip="https://www.screener.in/company/541865/"/>
-    <hyperlink ref="M64" r:id="rId126" tooltip="https://www.screener.in/company/541865/"/>
-    <hyperlink ref="B65" r:id="rId127" tooltip="https://www.screener.in/company/CBAZAAR/consolidated/"/>
-    <hyperlink ref="M65" r:id="rId128" tooltip="https://www.screener.in/company/CBAZAAR/consolidated/"/>
-    <hyperlink ref="B66" r:id="rId129" tooltip="https://www.screener.in/company/543521/"/>
-    <hyperlink ref="M66" r:id="rId130" tooltip="https://www.screener.in/company/543521/"/>
-    <hyperlink ref="B67" r:id="rId131" tooltip="https://www.screener.in/company/MKPL/"/>
-    <hyperlink ref="M67" r:id="rId132" tooltip="https://www.screener.in/company/MKPL/"/>
-    <hyperlink ref="B68" r:id="rId133" tooltip="https://www.screener.in/company/531153/"/>
-    <hyperlink ref="M68" r:id="rId134" tooltip="https://www.screener.in/company/531153/"/>
-    <hyperlink ref="B69" r:id="rId135" tooltip="https://www.screener.in/company/ZEELEARN/consolidated/"/>
-    <hyperlink ref="M69" r:id="rId136" tooltip="https://www.screener.in/company/ZEELEARN/consolidated/"/>
-    <hyperlink ref="B70" r:id="rId137" tooltip="https://www.screener.in/company/LCCINFOTEC/"/>
-    <hyperlink ref="M70" r:id="rId138" tooltip="https://www.screener.in/company/LCCINFOTEC/"/>
-    <hyperlink ref="B71" r:id="rId139" tooltip="https://www.screener.in/company/KEEPLEARN/"/>
-    <hyperlink ref="M71" r:id="rId140" tooltip="https://www.screener.in/company/KEEPLEARN/"/>
-    <hyperlink ref="B72" r:id="rId141" tooltip="https://www.screener.in/company/VIRTUALG/consolidated/"/>
-    <hyperlink ref="M72" r:id="rId142" tooltip="https://www.screener.in/company/VIRTUALG/consolidated/"/>
-    <hyperlink ref="B73" r:id="rId143" tooltip="https://www.screener.in/company/539761/"/>
-    <hyperlink ref="M73" r:id="rId144" tooltip="https://www.screener.in/company/539761/"/>
-    <hyperlink ref="B74" r:id="rId145" tooltip="https://www.screener.in/company/TREEHOUSE/consolidated/"/>
-    <hyperlink ref="M74" r:id="rId146" tooltip="https://www.screener.in/company/TREEHOUSE/consolidated/"/>
-    <hyperlink ref="B75" r:id="rId147" tooltip="https://www.screener.in/company/MTEDUCARE/consolidated/"/>
-    <hyperlink ref="M75" r:id="rId148" tooltip="https://www.screener.in/company/MTEDUCARE/consolidated/"/>
-    <hyperlink ref="B76" r:id="rId149" tooltip="https://www.screener.in/company/SAMBHAAV/consolidated/"/>
-    <hyperlink ref="M76" r:id="rId150" tooltip="https://www.screener.in/company/SAMBHAAV/consolidated/"/>
-    <hyperlink ref="B77" r:id="rId151" tooltip="https://www.screener.in/company/DNAMEDIA/"/>
-    <hyperlink ref="M77" r:id="rId152" tooltip="https://www.screener.in/company/DNAMEDIA/"/>
-    <hyperlink ref="B78" r:id="rId153" tooltip="https://www.screener.in/company/SHYAMCENT/"/>
-    <hyperlink ref="M78" r:id="rId154" tooltip="https://www.screener.in/company/SHYAMCENT/"/>
-    <hyperlink ref="B79" r:id="rId155" tooltip="https://www.screener.in/company/532656/consolidated/"/>
-    <hyperlink ref="M79" r:id="rId156" tooltip="https://www.screener.in/company/532656/consolidated/"/>
-    <hyperlink ref="B80" r:id="rId157" tooltip="https://www.screener.in/company/IMPEXFERRO/"/>
-    <hyperlink ref="M80" r:id="rId158" tooltip="https://www.screener.in/company/IMPEXFERRO/"/>
-    <hyperlink ref="B81" r:id="rId159" tooltip="https://www.screener.in/company/NAGAFERT/consolidated/"/>
-    <hyperlink ref="M81" r:id="rId160" tooltip="https://www.screener.in/company/NAGAFERT/consolidated/"/>
-    <hyperlink ref="B82" r:id="rId161" tooltip="https://www.screener.in/company/523277/consolidated/"/>
-    <hyperlink ref="M82" r:id="rId162" tooltip="https://www.screener.in/company/523277/consolidated/"/>
-    <hyperlink ref="B83" r:id="rId163" tooltip="https://www.screener.in/company/532355/consolidated/"/>
-    <hyperlink ref="M83" r:id="rId164" tooltip="https://www.screener.in/company/532355/consolidated/"/>
-    <hyperlink ref="B84" r:id="rId165" tooltip="https://www.screener.in/company/511092/"/>
-    <hyperlink ref="M84" r:id="rId166" tooltip="https://www.screener.in/company/511092/"/>
-    <hyperlink ref="B85" r:id="rId167" tooltip="https://www.screener.in/company/511246/"/>
-    <hyperlink ref="M85" r:id="rId168" tooltip="https://www.screener.in/company/511246/"/>
-    <hyperlink ref="B86" r:id="rId169" tooltip="https://www.screener.in/company/531512/"/>
-    <hyperlink ref="M86" r:id="rId170" tooltip="https://www.screener.in/company/531512/"/>
-    <hyperlink ref="B87" r:id="rId171" tooltip="https://www.screener.in/company/532072/"/>
-    <hyperlink ref="M87" r:id="rId172" tooltip="https://www.screener.in/company/532072/"/>
-    <hyperlink ref="B88" r:id="rId173" tooltip="https://www.screener.in/company/PPSL/consolidated/"/>
-    <hyperlink ref="M88" r:id="rId174" tooltip="https://www.screener.in/company/PPSL/consolidated/"/>
-    <hyperlink ref="B89" r:id="rId175" tooltip="https://www.screener.in/company/532160/"/>
-    <hyperlink ref="M89" r:id="rId176" tooltip="https://www.screener.in/company/532160/"/>
-    <hyperlink ref="B90" r:id="rId177" tooltip="https://www.screener.in/company/MOS/consolidated/"/>
-    <hyperlink ref="M90" r:id="rId178" tooltip="https://www.screener.in/company/MOS/consolidated/"/>
-    <hyperlink ref="B91" r:id="rId179" tooltip="https://www.screener.in/company/SUVIDHAA/consolidated/"/>
-    <hyperlink ref="M91" r:id="rId180" tooltip="https://www.screener.in/company/SUVIDHAA/consolidated/"/>
-    <hyperlink ref="B92" r:id="rId181" tooltip="https://www.screener.in/company/AGSTRA/consolidated/"/>
-    <hyperlink ref="M92" r:id="rId182" tooltip="https://www.screener.in/company/AGSTRA/consolidated/"/>
-    <hyperlink ref="B93" r:id="rId183" tooltip="https://www.screener.in/company/526490/"/>
-    <hyperlink ref="M93" r:id="rId184" tooltip="https://www.screener.in/company/526490/"/>
-    <hyperlink ref="B94" r:id="rId185" tooltip="https://www.screener.in/company/516062/"/>
-    <hyperlink ref="M94" r:id="rId186" tooltip="https://www.screener.in/company/516062/"/>
-    <hyperlink ref="B95" r:id="rId187" tooltip="https://www.screener.in/company/HARDWYN/"/>
-    <hyperlink ref="M95" r:id="rId188" tooltip="https://www.screener.in/company/HARDWYN/"/>
-    <hyperlink ref="B96" r:id="rId189" tooltip="https://www.screener.in/company/544188/"/>
-    <hyperlink ref="M96" r:id="rId190" tooltip="https://www.screener.in/company/544188/"/>
-    <hyperlink ref="B97" r:id="rId191" tooltip="https://www.screener.in/company/FILATFASH/consolidated/"/>
-    <hyperlink ref="M97" r:id="rId192" tooltip="https://www.screener.in/company/FILATFASH/consolidated/"/>
-    <hyperlink ref="B98" r:id="rId193" tooltip="https://www.screener.in/company/LAL/"/>
-    <hyperlink ref="M98" r:id="rId194" tooltip="https://www.screener.in/company/LAL/"/>
-    <hyperlink ref="B99" r:id="rId195" tooltip="https://www.screener.in/company/539216/consolidated/"/>
-    <hyperlink ref="M99" r:id="rId196" tooltip="https://www.screener.in/company/539216/consolidated/"/>
-    <hyperlink ref="B100" r:id="rId197" tooltip="https://www.screener.in/company/VINNY/"/>
-    <hyperlink ref="M100" r:id="rId198" tooltip="https://www.screener.in/company/VINNY/"/>
-    <hyperlink ref="B101" r:id="rId199" tooltip="https://www.screener.in/company/CELEBRITY/"/>
-    <hyperlink ref="M101" r:id="rId200" tooltip="https://www.screener.in/company/CELEBRITY/"/>
-    <hyperlink ref="B102" r:id="rId201" tooltip="https://www.screener.in/company/542579/"/>
-    <hyperlink ref="M102" r:id="rId202" tooltip="https://www.screener.in/company/542579/"/>
-    <hyperlink ref="B103" r:id="rId203" tooltip="https://www.screener.in/company/540252/"/>
-    <hyperlink ref="M103" r:id="rId204" tooltip="https://www.screener.in/company/540252/"/>
-    <hyperlink ref="B104" r:id="rId205" tooltip="https://www.screener.in/company/523373/consolidated/"/>
-    <hyperlink ref="M104" r:id="rId206" tooltip="https://www.screener.in/company/523373/consolidated/"/>
-    <hyperlink ref="B105" r:id="rId207" tooltip="https://www.screener.in/company/MOKSH/"/>
-    <hyperlink ref="M105" r:id="rId208" tooltip="https://www.screener.in/company/MOKSH/"/>
-    <hyperlink ref="B106" r:id="rId209" tooltip="https://www.screener.in/company/512047/"/>
-    <hyperlink ref="M106" r:id="rId210" tooltip="https://www.screener.in/company/512047/"/>
-    <hyperlink ref="B107" r:id="rId211" tooltip="https://www.screener.in/company/523387/consolidated/"/>
-    <hyperlink ref="M107" r:id="rId212" tooltip="https://www.screener.in/company/523387/consolidated/"/>
-    <hyperlink ref="B108" r:id="rId213" tooltip="https://www.screener.in/company/530525/"/>
-    <hyperlink ref="M108" r:id="rId214" tooltip="https://www.screener.in/company/530525/"/>
-    <hyperlink ref="B109" r:id="rId215" tooltip="https://www.screener.in/company/531626/"/>
-    <hyperlink ref="M109" r:id="rId216" tooltip="https://www.screener.in/company/531626/"/>
-    <hyperlink ref="B110" r:id="rId217" tooltip="https://www.screener.in/company/KANANIIND/consolidated/"/>
-    <hyperlink ref="M110" r:id="rId218" tooltip="https://www.screener.in/company/KANANIIND/consolidated/"/>
-    <hyperlink ref="B111" r:id="rId219" tooltip="https://www.screener.in/company/540953/"/>
-    <hyperlink ref="M111" r:id="rId220" tooltip="https://www.screener.in/company/540953/"/>
-    <hyperlink ref="B112" r:id="rId221" tooltip="https://www.screener.in/company/ORIENTALTL/"/>
-    <hyperlink ref="M112" r:id="rId222" tooltip="https://www.screener.in/company/ORIENTALTL/"/>
-    <hyperlink ref="B113" r:id="rId223" tooltip="https://www.screener.in/company/JYOTISTRUC/consolidated/"/>
-    <hyperlink ref="M113" r:id="rId224" tooltip="https://www.screener.in/company/JYOTISTRUC/consolidated/"/>
-    <hyperlink ref="B114" r:id="rId225" tooltip="https://www.screener.in/company/BILVYAPAR/consolidated/"/>
-    <hyperlink ref="M114" r:id="rId226" tooltip="https://www.screener.in/company/BILVYAPAR/consolidated/"/>
-    <hyperlink ref="B115" r:id="rId227" tooltip="https://www.screener.in/company/531658/consolidated/"/>
-    <hyperlink ref="M115" r:id="rId228" tooltip="https://www.screener.in/company/531658/consolidated/"/>
-    <hyperlink ref="B116" r:id="rId229" tooltip="https://www.screener.in/company/HLVLTD/"/>
-    <hyperlink ref="M116" r:id="rId230" tooltip="https://www.screener.in/company/HLVLTD/"/>
-    <hyperlink ref="B117" r:id="rId231" tooltip="https://www.screener.in/company/531663/"/>
-    <hyperlink ref="M117" r:id="rId232" tooltip="https://www.screener.in/company/531663/"/>
-    <hyperlink ref="B118" r:id="rId233" tooltip="https://www.screener.in/company/RHFL/"/>
-    <hyperlink ref="M118" r:id="rId234" tooltip="https://www.screener.in/company/RHFL/"/>
-    <hyperlink ref="B119" r:id="rId235" tooltip="https://www.screener.in/company/539017/"/>
-    <hyperlink ref="M119" r:id="rId236" tooltip="https://www.screener.in/company/539017/"/>
-    <hyperlink ref="B120" r:id="rId237" tooltip="https://www.screener.in/company/SALASAR/consolidated/"/>
-    <hyperlink ref="M120" r:id="rId238" tooltip="https://www.screener.in/company/SALASAR/consolidated/"/>
-    <hyperlink ref="B121" r:id="rId239" tooltip="https://www.screener.in/company/DPSCLTD/consolidated/"/>
-    <hyperlink ref="M121" r:id="rId240" tooltip="https://www.screener.in/company/DPSCLTD/consolidated/"/>
-    <hyperlink ref="B122" r:id="rId241" tooltip="https://www.screener.in/company/538765/"/>
-    <hyperlink ref="M122" r:id="rId242" tooltip="https://www.screener.in/company/538765/"/>
-    <hyperlink ref="B123" r:id="rId243" tooltip="https://www.screener.in/company/503663/"/>
-    <hyperlink ref="M123" r:id="rId244" tooltip="https://www.screener.in/company/503663/"/>
-    <hyperlink ref="B124" r:id="rId245" tooltip="https://www.screener.in/company/538451/"/>
-    <hyperlink ref="M124" r:id="rId246" tooltip="https://www.screener.in/company/538451/"/>
-    <hyperlink ref="B125" r:id="rId247" tooltip="https://www.screener.in/company/509051/"/>
-    <hyperlink ref="M125" r:id="rId248" tooltip="https://www.screener.in/company/509051/"/>
-    <hyperlink ref="B126" r:id="rId249" tooltip="https://www.screener.in/company/PARASPETRO/"/>
-    <hyperlink ref="M126" r:id="rId250" tooltip="https://www.screener.in/company/PARASPETRO/"/>
-    <hyperlink ref="B127" r:id="rId251" tooltip="https://www.screener.in/company/509053/consolidated/"/>
-    <hyperlink ref="M127" r:id="rId252" tooltip="https://www.screener.in/company/509053/consolidated/"/>
-    <hyperlink ref="B128" r:id="rId253" tooltip="https://www.screener.in/company/539091/"/>
-    <hyperlink ref="M128" r:id="rId254" tooltip="https://www.screener.in/company/539091/"/>
-    <hyperlink ref="B129" r:id="rId255" tooltip="https://www.screener.in/company/ANKITMETAL/"/>
-    <hyperlink ref="M129" r:id="rId256" tooltip="https://www.screener.in/company/ANKITMETAL/"/>
-    <hyperlink ref="B130" r:id="rId257" tooltip="https://www.screener.in/company/RAMASTEEL/consolidated/"/>
-    <hyperlink ref="M130" r:id="rId258" tooltip="https://www.screener.in/company/RAMASTEEL/consolidated/"/>
-    <hyperlink ref="B131" r:id="rId259" tooltip="https://www.screener.in/company/SHAH/consolidated/"/>
-    <hyperlink ref="M131" r:id="rId260" tooltip="https://www.screener.in/company/SHAH/consolidated/"/>
-    <hyperlink ref="B132" r:id="rId261" tooltip="https://www.screener.in/company/KRITIKA/"/>
-    <hyperlink ref="M132" r:id="rId262" tooltip="https://www.screener.in/company/KRITIKA/"/>
-    <hyperlink ref="B133" r:id="rId263" tooltip="https://www.screener.in/company/534064/"/>
-    <hyperlink ref="M133" r:id="rId264" tooltip="https://www.screener.in/company/534064/"/>
-    <hyperlink ref="B134" r:id="rId265" tooltip="https://www.screener.in/company/SUPREMEENG/"/>
-    <hyperlink ref="M134" r:id="rId266" tooltip="https://www.screener.in/company/SUPREMEENG/"/>
-    <hyperlink ref="B135" r:id="rId267" tooltip="https://www.screener.in/company/ZENITHSTL/consolidated/"/>
-    <hyperlink ref="M135" r:id="rId268" tooltip="https://www.screener.in/company/ZENITHSTL/consolidated/"/>
-    <hyperlink ref="B136" r:id="rId269" tooltip="https://www.screener.in/company/PRAKASHSTL/"/>
-    <hyperlink ref="M136" r:id="rId270" tooltip="https://www.screener.in/company/PRAKASHSTL/"/>
-    <hyperlink ref="B137" r:id="rId271" tooltip="https://www.screener.in/company/BCG/consolidated/"/>
-    <hyperlink ref="M137" r:id="rId272" tooltip="https://www.screener.in/company/BCG/consolidated/"/>
-    <hyperlink ref="B138" r:id="rId273" tooltip="https://www.screener.in/company/534535/consolidated/"/>
-    <hyperlink ref="M138" r:id="rId274" tooltip="https://www.screener.in/company/534535/consolidated/"/>
-    <hyperlink ref="B139" r:id="rId275" tooltip="https://www.screener.in/company/VAKRANGEE/consolidated/"/>
-    <hyperlink ref="M139" r:id="rId276" tooltip="https://www.screener.in/company/VAKRANGEE/consolidated/"/>
-    <hyperlink ref="B140" r:id="rId277" tooltip="https://www.screener.in/company/FCSSOFT/consolidated/"/>
-    <hyperlink ref="M140" r:id="rId278" tooltip="https://www.screener.in/company/FCSSOFT/consolidated/"/>
-    <hyperlink ref="B141" r:id="rId279" tooltip="https://www.screener.in/company/ASMS/consolidated/"/>
-    <hyperlink ref="M141" r:id="rId280" tooltip="https://www.screener.in/company/ASMS/consolidated/"/>
-    <hyperlink ref="B142" r:id="rId281" tooltip="https://www.screener.in/company/VLEGOV/"/>
-    <hyperlink ref="M142" r:id="rId282" tooltip="https://www.screener.in/company/VLEGOV/"/>
-    <hyperlink ref="B143" r:id="rId283" tooltip="https://www.screener.in/company/521005/"/>
-    <hyperlink ref="M143" r:id="rId284" tooltip="https://www.screener.in/company/521005/"/>
-    <hyperlink ref="B144" r:id="rId285" tooltip="https://www.screener.in/company/CRSL/"/>
-    <hyperlink ref="M144" r:id="rId286" tooltip="https://www.screener.in/company/CRSL/"/>
-    <hyperlink ref="B145" r:id="rId287" tooltip="https://www.screener.in/company/SGLRES/"/>
-    <hyperlink ref="M145" r:id="rId288" tooltip="https://www.screener.in/company/SGLRES/"/>
-    <hyperlink ref="B146" r:id="rId289" tooltip="https://www.screener.in/company/SUPTANERY/consolidated/"/>
-    <hyperlink ref="M146" r:id="rId290" tooltip="https://www.screener.in/company/SUPTANERY/consolidated/"/>
-    <hyperlink ref="B147" r:id="rId291" tooltip="https://www.screener.in/company/AKI/consolidated/"/>
-    <hyperlink ref="M147" r:id="rId292" tooltip="https://www.screener.in/company/AKI/consolidated/"/>
-    <hyperlink ref="B148" r:id="rId293" tooltip="https://www.screener.in/company/541771/"/>
-    <hyperlink ref="M148" r:id="rId294" tooltip="https://www.screener.in/company/541771/"/>
-    <hyperlink ref="B149" r:id="rId295" tooltip="https://www.screener.in/company/523242/"/>
-    <hyperlink ref="M149" r:id="rId296" tooltip="https://www.screener.in/company/523242/"/>
-    <hyperlink ref="B150" r:id="rId297" tooltip="https://www.screener.in/company/526415/consolidated/"/>
-    <hyperlink ref="M150" r:id="rId298" tooltip="https://www.screener.in/company/526415/consolidated/"/>
-    <hyperlink ref="B151" r:id="rId299" tooltip="https://www.screener.in/company/534190/"/>
-    <hyperlink ref="M151" r:id="rId300" tooltip="https://www.screener.in/company/534190/"/>
-    <hyperlink ref="B152" r:id="rId301" tooltip="https://www.screener.in/company/531977/"/>
-    <hyperlink ref="M152" r:id="rId302" tooltip="https://www.screener.in/company/531977/"/>
-    <hyperlink ref="B153" r:id="rId303" tooltip="https://www.screener.in/company/RADIOCITY/"/>
-    <hyperlink ref="M153" r:id="rId304" tooltip="https://www.screener.in/company/RADIOCITY/"/>
-    <hyperlink ref="B154" r:id="rId305" tooltip="https://www.screener.in/company/539175/"/>
-    <hyperlink ref="M154" r:id="rId306" tooltip="https://www.screener.in/company/539175/"/>
-    <hyperlink ref="B155" r:id="rId307" tooltip="https://www.screener.in/company/STUDIOLSD/"/>
-    <hyperlink ref="M155" r:id="rId308" tooltip="https://www.screener.in/company/STUDIOLSD/"/>
-    <hyperlink ref="B156" r:id="rId309" tooltip="https://www.screener.in/company/NEXTMEDIA/"/>
-    <hyperlink ref="M156" r:id="rId310" tooltip="https://www.screener.in/company/NEXTMEDIA/"/>
-    <hyperlink ref="B157" r:id="rId311" tooltip="https://www.screener.in/company/512499/"/>
-    <hyperlink ref="M157" r:id="rId312" tooltip="https://www.screener.in/company/512499/"/>
-    <hyperlink ref="B158" r:id="rId313" tooltip="https://www.screener.in/company/RADAAN/consolidated/"/>
-    <hyperlink ref="M158" r:id="rId314" tooltip="https://www.screener.in/company/RADAAN/consolidated/"/>
-    <hyperlink ref="B159" r:id="rId315" tooltip="https://www.screener.in/company/INSPIRE/"/>
-    <hyperlink ref="M159" r:id="rId316" tooltip="https://www.screener.in/company/INSPIRE/"/>
-    <hyperlink ref="B160" r:id="rId317" tooltip="https://www.screener.in/company/CREATIVEYE/"/>
-    <hyperlink ref="M160" r:id="rId318" tooltip="https://www.screener.in/company/CREATIVEYE/"/>
-    <hyperlink ref="B161" r:id="rId319" tooltip="https://www.screener.in/company/501945/"/>
-    <hyperlink ref="M161" r:id="rId320" tooltip="https://www.screener.in/company/501945/"/>
-    <hyperlink ref="B162" r:id="rId321" tooltip="https://www.screener.in/company/AFIL/"/>
-    <hyperlink ref="M162" r:id="rId322" tooltip="https://www.screener.in/company/AFIL/"/>
-    <hyperlink ref="B163" r:id="rId323" tooltip="https://www.screener.in/company/532320/consolidated/"/>
-    <hyperlink ref="M163" r:id="rId324" tooltip="https://www.screener.in/company/532320/consolidated/"/>
-    <hyperlink ref="B164" r:id="rId325" tooltip="https://www.screener.in/company/532275/"/>
-    <hyperlink ref="M164" r:id="rId326" tooltip="https://www.screener.in/company/532275/"/>
-    <hyperlink ref="B165" r:id="rId327" tooltip="https://www.screener.in/company/526961/consolidated/"/>
-    <hyperlink ref="M165" r:id="rId328" tooltip="https://www.screener.in/company/526961/consolidated/"/>
-    <hyperlink ref="B166" r:id="rId329" tooltip="https://www.screener.in/company/534060/"/>
-    <hyperlink ref="M166" r:id="rId330" tooltip="https://www.screener.in/company/534060/"/>
-    <hyperlink ref="B167" r:id="rId331" tooltip="https://www.screener.in/company/507962/"/>
-    <hyperlink ref="M167" r:id="rId332" tooltip="https://www.screener.in/company/507962/"/>
-    <hyperlink ref="B168" r:id="rId333" tooltip="https://www.screener.in/company/530557/"/>
-    <hyperlink ref="M168" r:id="rId334" tooltip="https://www.screener.in/company/530557/"/>
-    <hyperlink ref="B169" r:id="rId335" tooltip="https://www.screener.in/company/538860/"/>
-    <hyperlink ref="M169" r:id="rId336" tooltip="https://www.screener.in/company/538860/"/>
-    <hyperlink ref="B170" r:id="rId337" tooltip="https://www.screener.in/company/AAKASH/"/>
-    <hyperlink ref="M170" r:id="rId338" tooltip="https://www.screener.in/company/AAKASH/"/>
-    <hyperlink ref="B171" r:id="rId339" tooltip="https://www.screener.in/company/SARVESHWAR/consolidated/"/>
-    <hyperlink ref="M171" r:id="rId340" tooltip="https://www.screener.in/company/SARVESHWAR/consolidated/"/>
-    <hyperlink ref="B172" r:id="rId341" tooltip="https://www.screener.in/company/526445/consolidated/"/>
-    <hyperlink ref="M172" r:id="rId342" tooltip="https://www.screener.in/company/526445/consolidated/"/>
-    <hyperlink ref="B173" r:id="rId343" tooltip="https://www.screener.in/company/526899/"/>
-    <hyperlink ref="M173" r:id="rId344" tooltip="https://www.screener.in/company/526899/"/>
-    <hyperlink ref="B174" r:id="rId345" tooltip="https://www.screener.in/company/523467/"/>
-    <hyperlink ref="M174" r:id="rId346" tooltip="https://www.screener.in/company/523467/"/>
-    <hyperlink ref="B175" r:id="rId347" tooltip="https://www.screener.in/company/URJA/consolidated/"/>
-    <hyperlink ref="M175" r:id="rId348" tooltip="https://www.screener.in/company/URJA/consolidated/"/>
-    <hyperlink ref="B176" r:id="rId349" tooltip="https://www.screener.in/company/DELPHIFX/consolidated/"/>
-    <hyperlink ref="M176" r:id="rId350" tooltip="https://www.screener.in/company/DELPHIFX/consolidated/"/>
-    <hyperlink ref="B177" r:id="rId351" tooltip="https://www.screener.in/company/GATECH/"/>
-    <hyperlink ref="M177" r:id="rId352" tooltip="https://www.screener.in/company/GATECH/"/>
-    <hyperlink ref="B178" r:id="rId353" tooltip="https://www.screener.in/company/512018/consolidated/"/>
-    <hyperlink ref="M178" r:id="rId354" tooltip="https://www.screener.in/company/512018/consolidated/"/>
-    <hyperlink ref="B179" r:id="rId355" tooltip="https://www.screener.in/company/530881/"/>
-    <hyperlink ref="M179" r:id="rId356" tooltip="https://www.screener.in/company/530881/"/>
-    <hyperlink ref="B180" r:id="rId357" tooltip="https://www.screener.in/company/531950/consolidated/"/>
-    <hyperlink ref="M180" r:id="rId358" tooltip="https://www.screener.in/company/531950/consolidated/"/>
-    <hyperlink ref="B181" r:id="rId359" tooltip="https://www.screener.in/company/539132/"/>
-    <hyperlink ref="M181" r:id="rId360" tooltip="https://www.screener.in/company/539132/"/>
-    <hyperlink ref="B182" r:id="rId361" tooltip="https://www.screener.in/company/517554/consolidated/"/>
-    <hyperlink ref="M182" r:id="rId362" tooltip="https://www.screener.in/company/517554/consolidated/"/>
-    <hyperlink ref="B183" r:id="rId363" tooltip="https://www.screener.in/company/524614/"/>
-    <hyperlink ref="M183" r:id="rId364" tooltip="https://www.screener.in/company/524614/"/>
-    <hyperlink ref="B184" r:id="rId365" tooltip="https://www.screener.in/company/SANWARIA/consolidated/"/>
-    <hyperlink ref="M184" r:id="rId366" tooltip="https://www.screener.in/company/SANWARIA/consolidated/"/>
-    <hyperlink ref="B185" r:id="rId367" tooltip="https://www.screener.in/company/531716/"/>
-    <hyperlink ref="M185" r:id="rId368" tooltip="https://www.screener.in/company/531716/"/>
-    <hyperlink ref="B186" r:id="rId369" tooltip="https://www.screener.in/company/539219/consolidated/"/>
-    <hyperlink ref="M186" r:id="rId370" tooltip="https://www.screener.in/company/539219/consolidated/"/>
-    <hyperlink ref="B187" r:id="rId371" tooltip="https://www.screener.in/company/GTL/"/>
-    <hyperlink ref="M187" r:id="rId372" tooltip="https://www.screener.in/company/GTL/"/>
-    <hyperlink ref="B188" r:id="rId373" tooltip="https://www.screener.in/company/ALOKINDS/consolidated/"/>
-    <hyperlink ref="M188" r:id="rId374" tooltip="https://www.screener.in/company/ALOKINDS/consolidated/"/>
-    <hyperlink ref="B189" r:id="rId375" tooltip="https://www.screener.in/company/NDL/"/>
-    <hyperlink ref="M189" r:id="rId376" tooltip="https://www.screener.in/company/NDL/"/>
-    <hyperlink ref="B190" r:id="rId377" tooltip="https://www.screener.in/company/AXITA/"/>
-    <hyperlink ref="M190" r:id="rId378" tooltip="https://www.screener.in/company/AXITA/"/>
-    <hyperlink ref="B191" r:id="rId379" tooltip="https://www.screener.in/company/VARDMNPOLY/"/>
-    <hyperlink ref="M191" r:id="rId380" tooltip="https://www.screener.in/company/VARDMNPOLY/"/>
-    <hyperlink ref="B192" r:id="rId381" tooltip="https://www.screener.in/company/RNBDENIMS/consolidated/"/>
-    <hyperlink ref="M192" r:id="rId382" tooltip="https://www.screener.in/company/RNBDENIMS/consolidated/"/>
-    <hyperlink ref="B193" r:id="rId383" tooltip="https://www.screener.in/company/TTL/"/>
-    <hyperlink ref="M193" r:id="rId384" tooltip="https://www.screener.in/company/TTL/"/>
-    <hyperlink ref="B194" r:id="rId385" tooltip="https://www.screener.in/company/531411/"/>
-    <hyperlink ref="M194" r:id="rId386" tooltip="https://www.screener.in/company/531411/"/>
-    <hyperlink ref="B195" r:id="rId387" tooltip="https://www.screener.in/company/530185/"/>
-    <hyperlink ref="M195" r:id="rId388" tooltip="https://www.screener.in/company/530185/"/>
-    <hyperlink ref="B196" r:id="rId389" tooltip="https://www.screener.in/company/GLOBE/consolidated/"/>
-    <hyperlink ref="M196" r:id="rId390" tooltip="https://www.screener.in/company/GLOBE/consolidated/"/>
-    <hyperlink ref="B197" r:id="rId391" tooltip="https://www.screener.in/company/BHANDARI/"/>
-    <hyperlink ref="M197" r:id="rId392" tooltip="https://www.screener.in/company/BHANDARI/"/>
-    <hyperlink ref="B198" r:id="rId393" tooltip="https://www.screener.in/company/539594/consolidated/"/>
-    <hyperlink ref="M198" r:id="rId394" tooltip="https://www.screener.in/company/539594/consolidated/"/>
-    <hyperlink ref="B199" r:id="rId395" tooltip="https://www.screener.in/company/530617/"/>
-    <hyperlink ref="M199" r:id="rId396" tooltip="https://www.screener.in/company/530617/"/>
-    <hyperlink ref="B200" r:id="rId397" tooltip="https://www.screener.in/company/DANGEE/"/>
-    <hyperlink ref="M200" r:id="rId398" tooltip="https://www.screener.in/company/DANGEE/"/>
-    <hyperlink ref="B201" r:id="rId399" tooltip="https://www.screener.in/company/530217/"/>
-    <hyperlink ref="M201" r:id="rId400" tooltip="https://www.screener.in/company/530217/"/>
-    <hyperlink ref="B202" r:id="rId401" tooltip="https://www.screener.in/company/538520/"/>
-    <hyperlink ref="M202" r:id="rId402" tooltip="https://www.screener.in/company/538520/"/>
-    <hyperlink ref="B203" r:id="rId403" tooltip="https://www.screener.in/company/519500/"/>
-    <hyperlink ref="M203" r:id="rId404" tooltip="https://www.screener.in/company/519500/"/>
-    <hyperlink ref="B204" r:id="rId405" tooltip="https://www.screener.in/company/523105/"/>
-    <hyperlink ref="M204" r:id="rId406" tooltip="https://www.screener.in/company/523105/"/>
-    <hyperlink ref="B205" r:id="rId407" tooltip="https://www.screener.in/company/ROLLT/consolidated/"/>
-    <hyperlink ref="M205" r:id="rId408" tooltip="https://www.screener.in/company/ROLLT/consolidated/"/>
-    <hyperlink ref="B206" r:id="rId409" tooltip="https://www.screener.in/company/KAMOPAINTS/consolidated/"/>
-    <hyperlink ref="M206" r:id="rId410" tooltip="https://www.screener.in/company/KAMOPAINTS/consolidated/"/>
-    <hyperlink ref="B207" r:id="rId411" tooltip="https://www.screener.in/company/543579/"/>
-    <hyperlink ref="M207" r:id="rId412" tooltip="https://www.screener.in/company/543579/"/>
-    <hyperlink ref="B208" r:id="rId413" tooltip="https://www.screener.in/company/SIKKO/"/>
-    <hyperlink ref="M208" r:id="rId414" tooltip="https://www.screener.in/company/SIKKO/"/>
-    <hyperlink ref="B209" r:id="rId415" tooltip="https://www.screener.in/company/514165/consolidated/"/>
-    <hyperlink ref="M209" r:id="rId416" tooltip="https://www.screener.in/company/514165/consolidated/"/>
-    <hyperlink ref="B210" r:id="rId417" tooltip="https://www.screener.in/company/530027/"/>
-    <hyperlink ref="M210" r:id="rId418" tooltip="https://www.screener.in/company/530027/"/>
-    <hyperlink ref="B211" r:id="rId419" tooltip="https://www.screener.in/company/531739/consolidated/"/>
-    <hyperlink ref="M211" r:id="rId420" tooltip="https://www.screener.in/company/531739/consolidated/"/>
-    <hyperlink ref="B212" r:id="rId421" tooltip="https://www.screener.in/company/543499/"/>
-    <hyperlink ref="M212" r:id="rId422" tooltip="https://www.screener.in/company/543499/"/>
-    <hyperlink ref="B213" r:id="rId423" tooltip="https://www.screener.in/company/524238/"/>
-    <hyperlink ref="M213" r:id="rId424" tooltip="https://www.screener.in/company/524238/"/>
-    <hyperlink ref="B214" r:id="rId425" tooltip="https://www.screener.in/company/PILITA/"/>
-    <hyperlink ref="M214" r:id="rId426" tooltip="https://www.screener.in/company/PILITA/"/>
-    <hyperlink ref="B215" r:id="rId427" tooltip="https://www.screener.in/company/AVROIND/"/>
-    <hyperlink ref="M215" r:id="rId428" tooltip="https://www.screener.in/company/AVROIND/"/>
-    <hyperlink ref="B216" r:id="rId429" tooltip="https://www.screener.in/company/538817/consolidated/"/>
-    <hyperlink ref="M216" r:id="rId430" tooltip="https://www.screener.in/company/538817/consolidated/"/>
-    <hyperlink ref="B217" r:id="rId431" tooltip="https://www.screener.in/company/513337/consolidated/"/>
-    <hyperlink ref="M217" r:id="rId432" tooltip="https://www.screener.in/company/513337/consolidated/"/>
-    <hyperlink ref="B218" r:id="rId433" tooltip="https://www.screener.in/company/RTNPOWER/consolidated/"/>
-    <hyperlink ref="M218" r:id="rId434" tooltip="https://www.screener.in/company/RTNPOWER/consolidated/"/>
-    <hyperlink ref="B219" r:id="rId435" tooltip="https://www.screener.in/company/GREENPOWER/consolidated/"/>
-    <hyperlink ref="M219" r:id="rId436" tooltip="https://www.screener.in/company/GREENPOWER/consolidated/"/>
-    <hyperlink ref="B220" r:id="rId437" tooltip="https://www.screener.in/company/GVKPIL/consolidated/"/>
-    <hyperlink ref="M220" r:id="rId438" tooltip="https://www.screener.in/company/GVKPIL/consolidated/"/>
-    <hyperlink ref="B221" r:id="rId439" tooltip="https://www.screener.in/company/INDOWIND/consolidated/"/>
-    <hyperlink ref="M221" r:id="rId440" tooltip="https://www.screener.in/company/INDOWIND/consolidated/"/>
-    <hyperlink ref="B222" r:id="rId441" tooltip="https://www.screener.in/company/500014/"/>
-    <hyperlink ref="M222" r:id="rId442" tooltip="https://www.screener.in/company/500014/"/>
-    <hyperlink ref="B223" r:id="rId443" tooltip="https://www.screener.in/company/INFOMEDIA/"/>
-    <hyperlink ref="M223" r:id="rId444" tooltip="https://www.screener.in/company/INFOMEDIA/"/>
-    <hyperlink ref="B224" r:id="rId445" tooltip="https://www.screener.in/company/526841/"/>
-    <hyperlink ref="M224" r:id="rId446" tooltip="https://www.screener.in/company/526841/"/>
-    <hyperlink ref="B225" r:id="rId447" tooltip="https://www.screener.in/company/KSHITIJPOL/consolidated/"/>
-    <hyperlink ref="M225" r:id="rId448" tooltip="https://www.screener.in/company/KSHITIJPOL/consolidated/"/>
-    <hyperlink ref="B226" r:id="rId449" tooltip="https://www.screener.in/company/LPDC/"/>
-    <hyperlink ref="M226" r:id="rId450" tooltip="https://www.screener.in/company/LPDC/"/>
-    <hyperlink ref="B227" r:id="rId451" tooltip="https://www.screener.in/company/530053/"/>
-    <hyperlink ref="M227" r:id="rId452" tooltip="https://www.screener.in/company/530053/"/>
-    <hyperlink ref="B228" r:id="rId453" tooltip="https://www.screener.in/company/543400/"/>
-    <hyperlink ref="M228" r:id="rId454" tooltip="https://www.screener.in/company/543400/"/>
-    <hyperlink ref="B229" r:id="rId455" tooltip="https://www.screener.in/company/UNITECH/consolidated/"/>
-    <hyperlink ref="M229" r:id="rId456" tooltip="https://www.screener.in/company/UNITECH/consolidated/"/>
-    <hyperlink ref="B230" r:id="rId457" tooltip="https://www.screener.in/company/NILAINFRA/consolidated/"/>
-    <hyperlink ref="M230" r:id="rId458" tooltip="https://www.screener.in/company/NILAINFRA/consolidated/"/>
-    <hyperlink ref="B231" r:id="rId459" tooltip="https://www.screener.in/company/HAMPTON/consolidated/"/>
-    <hyperlink ref="M231" r:id="rId460" tooltip="https://www.screener.in/company/HAMPTON/consolidated/"/>
-    <hyperlink ref="B232" r:id="rId461" tooltip="https://www.screener.in/company/PARSVNATH/consolidated/"/>
-    <hyperlink ref="M232" r:id="rId462" tooltip="https://www.screener.in/company/PARSVNATH/consolidated/"/>
-    <hyperlink ref="B233" r:id="rId463" tooltip="https://www.screener.in/company/531273/"/>
-    <hyperlink ref="M233" r:id="rId464" tooltip="https://www.screener.in/company/531273/"/>
-    <hyperlink ref="B234" r:id="rId465" tooltip="https://www.screener.in/company/NOIDATOLL/consolidated/"/>
-    <hyperlink ref="M234" r:id="rId466" tooltip="https://www.screener.in/company/NOIDATOLL/consolidated/"/>
-    <hyperlink ref="B235" r:id="rId467" tooltip="https://www.screener.in/company/GAYAHWS/consolidated/"/>
-    <hyperlink ref="M235" r:id="rId468" tooltip="https://www.screener.in/company/GAYAHWS/consolidated/"/>
-    <hyperlink ref="B236" r:id="rId469" tooltip="https://www.screener.in/company/MEP/"/>
-    <hyperlink ref="M236" r:id="rId470" tooltip="https://www.screener.in/company/MEP/"/>
-    <hyperlink ref="B237" r:id="rId471" tooltip="https://www.screener.in/company/526795/"/>
-    <hyperlink ref="M237" r:id="rId472" tooltip="https://www.screener.in/company/526795/"/>
-    <hyperlink ref="B238" r:id="rId473" tooltip="https://www.screener.in/company/AVANCE/consolidated/"/>
-    <hyperlink ref="M238" r:id="rId474" tooltip="https://www.screener.in/company/AVANCE/consolidated/"/>
-    <hyperlink ref="B239" r:id="rId475" tooltip="https://www.screener.in/company/512093/consolidated/"/>
-    <hyperlink ref="M239" r:id="rId476" tooltip="https://www.screener.in/company/512093/consolidated/"/>
-    <hyperlink ref="B240" r:id="rId477" tooltip="https://www.screener.in/company/PRAXIS/"/>
-    <hyperlink ref="M240" r:id="rId478" tooltip="https://www.screener.in/company/PRAXIS/"/>
-    <hyperlink ref="B241" r:id="rId479" tooltip="https://www.screener.in/company/540615/"/>
-    <hyperlink ref="M241" r:id="rId480" tooltip="https://www.screener.in/company/540615/"/>
-    <hyperlink ref="B242" r:id="rId481" tooltip="https://www.screener.in/company/VIKASECO/consolidated/"/>
-    <hyperlink ref="M242" r:id="rId482" tooltip="https://www.screener.in/company/VIKASECO/consolidated/"/>
-    <hyperlink ref="B243" r:id="rId483" tooltip="https://www.screener.in/company/SUNDARAM/"/>
-    <hyperlink ref="M243" r:id="rId484" tooltip="https://www.screener.in/company/SUNDARAM/"/>
-    <hyperlink ref="B244" r:id="rId485" tooltip="https://www.screener.in/company/539228/"/>
-    <hyperlink ref="M244" r:id="rId486" tooltip="https://www.screener.in/company/539228/"/>
-    <hyperlink ref="B245" r:id="rId487" tooltip="https://www.screener.in/company/VASA/"/>
-    <hyperlink ref="M245" r:id="rId488" tooltip="https://www.screener.in/company/VASA/"/>
-    <hyperlink ref="B246" r:id="rId489" tooltip="https://www.screener.in/company/INVENTURE/consolidated/"/>
-    <hyperlink ref="M246" r:id="rId490" tooltip="https://www.screener.in/company/INVENTURE/consolidated/"/>
-    <hyperlink ref="B247" r:id="rId491" tooltip="https://www.screener.in/company/535431/"/>
-    <hyperlink ref="M247" r:id="rId492" tooltip="https://www.screener.in/company/535431/"/>
-    <hyperlink ref="B248" r:id="rId493" tooltip="https://www.screener.in/company/VISHWARAJ/"/>
-    <hyperlink ref="M248" r:id="rId494" tooltip="https://www.screener.in/company/VISHWARAJ/"/>
-    <hyperlink ref="B249" r:id="rId495" tooltip="https://www.screener.in/company/541347/"/>
-    <hyperlink ref="M249" r:id="rId496" tooltip="https://www.screener.in/company/541347/"/>
-    <hyperlink ref="B250" r:id="rId497" tooltip="https://www.screener.in/company/532183/"/>
-    <hyperlink ref="M250" r:id="rId498" tooltip="https://www.screener.in/company/532183/"/>
-    <hyperlink ref="B251" r:id="rId499" tooltip="https://www.screener.in/company/SIMBHALS/consolidated/"/>
-    <hyperlink ref="M251" r:id="rId500" tooltip="https://www.screener.in/company/SIMBHALS/consolidated/"/>
-    <hyperlink ref="B252" r:id="rId501" tooltip="https://www.screener.in/company/537709/"/>
-    <hyperlink ref="M252" r:id="rId502" tooltip="https://www.screener.in/company/537709/"/>
-    <hyperlink ref="B253" r:id="rId503" tooltip="https://www.screener.in/company/AKSHOPTFBR/consolidated/"/>
-    <hyperlink ref="M253" r:id="rId504" tooltip="https://www.screener.in/company/AKSHOPTFBR/consolidated/"/>
-    <hyperlink ref="B254" r:id="rId505" tooltip="https://www.screener.in/company/532975/"/>
-    <hyperlink ref="M254" r:id="rId506" tooltip="https://www.screener.in/company/532975/"/>
-    <hyperlink ref="B255" r:id="rId507" tooltip="https://www.screener.in/company/RCOM/consolidated/"/>
-    <hyperlink ref="M255" r:id="rId508" tooltip="https://www.screener.in/company/RCOM/consolidated/"/>
-    <hyperlink ref="B256" r:id="rId509" tooltip="https://www.screener.in/company/511116/"/>
-    <hyperlink ref="M256" r:id="rId510" tooltip="https://www.screener.in/company/511116/"/>
-    <hyperlink ref="B257" r:id="rId511" tooltip="https://www.screener.in/company/538674/"/>
-    <hyperlink ref="M257" r:id="rId512" tooltip="https://www.screener.in/company/538674/"/>
-    <hyperlink ref="B258" r:id="rId513" tooltip="https://www.screener.in/company/GTLINFRA/"/>
-    <hyperlink ref="M258" r:id="rId514" tooltip="https://www.screener.in/company/GTLINFRA/"/>
-    <hyperlink ref="B259" r:id="rId515" tooltip="https://www.screener.in/company/EASEMYTRIP/consolidated/"/>
-    <hyperlink ref="M259" r:id="rId516" tooltip="https://www.screener.in/company/EASEMYTRIP/consolidated/"/>
-    <hyperlink ref="B260" r:id="rId517" tooltip="https://www.screener.in/company/544242/"/>
-    <hyperlink ref="M260" r:id="rId518" tooltip="https://www.screener.in/company/544242/"/>
-    <hyperlink ref="B261" r:id="rId519" tooltip="https://www.screener.in/company/543541/"/>
-    <hyperlink ref="M261" r:id="rId520" tooltip="https://www.screener.in/company/543541/"/>
-    <hyperlink ref="B262" r:id="rId521" tooltip="https://www.screener.in/company/524444/consolidated/"/>
-    <hyperlink ref="M262" r:id="rId522" tooltip="https://www.screener.in/company/524444/consolidated/"/>
-    <hyperlink ref="B263" r:id="rId523" tooltip="https://www.screener.in/company/542012/"/>
-    <hyperlink ref="M263" r:id="rId524" tooltip="https://www.screener.in/company/542012/"/>
-    <hyperlink ref="B264" r:id="rId525" tooltip="https://www.screener.in/company/539800/"/>
-    <hyperlink ref="M264" r:id="rId526" tooltip="https://www.screener.in/company/539800/"/>
-    <hyperlink ref="B265" r:id="rId527" tooltip="https://www.screener.in/company/543798/"/>
-    <hyperlink ref="M265" r:id="rId528" tooltip="https://www.screener.in/company/543798/"/>
-    <hyperlink ref="B266" r:id="rId529" tooltip="https://www.screener.in/company/540492/"/>
-    <hyperlink ref="M266" r:id="rId530" tooltip="https://www.screener.in/company/540492/"/>
-    <hyperlink ref="B267" r:id="rId531" tooltip="https://www.screener.in/company/HEADSUP/"/>
-    <hyperlink ref="M267" r:id="rId532" tooltip="https://www.screener.in/company/HEADSUP/"/>
-    <hyperlink ref="B268" r:id="rId533" tooltip="https://www.screener.in/company/542206/"/>
-    <hyperlink ref="M268" r:id="rId534" tooltip="https://www.screener.in/company/542206/"/>
-    <hyperlink ref="B269" r:id="rId535" tooltip="https://www.screener.in/company/540717/consolidated/"/>
-    <hyperlink ref="M269" r:id="rId536" tooltip="https://www.screener.in/company/540717/consolidated/"/>
-    <hyperlink ref="B270" r:id="rId537" tooltip="https://www.screener.in/company/SAKUMA/consolidated/"/>
-    <hyperlink ref="M270" r:id="rId538" tooltip="https://www.screener.in/company/SAKUMA/consolidated/"/>
-    <hyperlink ref="B271" r:id="rId539" tooltip="https://www.screener.in/company/VIKASLIFE/consolidated/"/>
-    <hyperlink ref="M271" r:id="rId540" tooltip="https://www.screener.in/company/VIKASLIFE/consolidated/"/>
-    <hyperlink ref="B272" r:id="rId541" tooltip="https://www.screener.in/company/SPCENET/consolidated/"/>
-    <hyperlink ref="M272" r:id="rId542" tooltip="https://www.screener.in/company/SPCENET/consolidated/"/>
-    <hyperlink ref="B273" r:id="rId543" tooltip="https://www.screener.in/company/ESSENTIA/consolidated/"/>
-    <hyperlink ref="M273" r:id="rId544" tooltip="https://www.screener.in/company/ESSENTIA/consolidated/"/>
-    <hyperlink ref="B274" r:id="rId545" tooltip="https://www.screener.in/company/LANDSMILL/consolidated/"/>
-    <hyperlink ref="M274" r:id="rId546" tooltip="https://www.screener.in/company/LANDSMILL/consolidated/"/>
-    <hyperlink ref="B275" r:id="rId547" tooltip="https://www.screener.in/company/HATHWAY/consolidated/"/>
-    <hyperlink ref="M275" r:id="rId548" tooltip="https://www.screener.in/company/HATHWAY/consolidated/"/>
-    <hyperlink ref="B276" r:id="rId549" tooltip="https://www.screener.in/company/ZEEMEDIA/consolidated/"/>
-    <hyperlink ref="M276" r:id="rId550" tooltip="https://www.screener.in/company/ZEEMEDIA/consolidated/"/>
-    <hyperlink ref="B277" r:id="rId551" tooltip="https://www.screener.in/company/DISHTV/consolidated/"/>
-    <hyperlink ref="M277" r:id="rId552" tooltip="https://www.screener.in/company/DISHTV/consolidated/"/>
-    <hyperlink ref="B278" r:id="rId553" tooltip="https://www.screener.in/company/BAGFILMS/consolidated/"/>
-    <hyperlink ref="M278" r:id="rId554" tooltip="https://www.screener.in/company/BAGFILMS/consolidated/"/>
-    <hyperlink ref="B279" r:id="rId555" tooltip="https://www.screener.in/company/SITINET/consolidated/"/>
-    <hyperlink ref="M279" r:id="rId556" tooltip="https://www.screener.in/company/SITINET/consolidated/"/>
-    <hyperlink ref="B280" r:id="rId557" tooltip="https://www.screener.in/company/540821/"/>
-    <hyperlink ref="M280" r:id="rId558" tooltip="https://www.screener.in/company/540821/"/>
-    <hyperlink ref="B281" r:id="rId559" tooltip="https://www.screener.in/company/521062/"/>
-    <hyperlink ref="M281" r:id="rId560" tooltip="https://www.screener.in/company/521062/"/>
-    <hyperlink ref="B282" r:id="rId561" tooltip="https://www.screener.in/company/TVVISION/consolidated/"/>
-    <hyperlink ref="M282" r:id="rId562" tooltip="https://www.screener.in/company/TVVISION/consolidated/"/>
-    <hyperlink ref="B283" r:id="rId563" tooltip="https://www.screener.in/company/ORTEL/"/>
-    <hyperlink ref="M283" r:id="rId564" tooltip="https://www.screener.in/company/ORTEL/"/>
-    <hyperlink ref="B284" r:id="rId565" tooltip="https://www.screener.in/company/533268/consolidated/"/>
-    <hyperlink ref="M284" r:id="rId566" tooltip="https://www.screener.in/company/533268/consolidated/"/>
-    <hyperlink ref="B285" r:id="rId567" tooltip="https://www.screener.in/company/539040/"/>
-    <hyperlink ref="M285" r:id="rId568" tooltip="https://www.screener.in/company/539040/"/>
+    <hyperlink ref="B2" r:id="rId1" tooltip="https://www.screener.in/company/WARDINMOBI/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="M2" r:id="rId2" tooltip="https://www.screener.in/company/WARDINMOBI/" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B3" r:id="rId3" tooltip="https://www.screener.in/company/539310/" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="M3" r:id="rId4" tooltip="https://www.screener.in/company/539310/" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="B4" r:id="rId5" tooltip="https://www.screener.in/company/543341/consolidated/" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="M4" r:id="rId6" tooltip="https://www.screener.in/company/543341/consolidated/" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B5" r:id="rId7" tooltip="https://www.screener.in/company/526441/consolidated/" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="M5" r:id="rId8" tooltip="https://www.screener.in/company/526441/consolidated/" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B6" r:id="rId9" tooltip="https://www.screener.in/company/SPICEJET/" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="M6" r:id="rId10" tooltip="https://www.screener.in/company/SPICEJET/" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="B7" r:id="rId11" tooltip="https://www.screener.in/company/531869/" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="M7" r:id="rId12" tooltip="https://www.screener.in/company/531869/" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="B8" r:id="rId13" tooltip="https://www.screener.in/company/513502/" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="M8" r:id="rId14" tooltip="https://www.screener.in/company/513502/" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B9" r:id="rId15" tooltip="https://www.screener.in/company/RAJMET/" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="M9" r:id="rId16" tooltip="https://www.screener.in/company/RAJMET/" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B10" r:id="rId17" tooltip="https://www.screener.in/company/538731/" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="M10" r:id="rId18" tooltip="https://www.screener.in/company/538731/" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B11" r:id="rId19" tooltip="https://www.screener.in/company/AJOONI/" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="M11" r:id="rId20" tooltip="https://www.screener.in/company/AJOONI/" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B12" r:id="rId21" tooltip="https://www.screener.in/company/IVC/consolidated/" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="M12" r:id="rId22" tooltip="https://www.screener.in/company/IVC/consolidated/" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="B13" r:id="rId23" tooltip="https://www.screener.in/company/539402/" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="M13" r:id="rId24" tooltip="https://www.screener.in/company/539402/" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="B14" r:id="rId25" tooltip="https://www.screener.in/company/539470/" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="M14" r:id="rId26" tooltip="https://www.screener.in/company/539470/" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="B15" r:id="rId27" tooltip="https://www.screener.in/company/COMFINTE/consolidated/" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="M15" r:id="rId28" tooltip="https://www.screener.in/company/COMFINTE/consolidated/" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="B16" r:id="rId29" tooltip="https://www.screener.in/company/532139/" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="M16" r:id="rId30" tooltip="https://www.screener.in/company/532139/" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="B17" r:id="rId31" tooltip="https://www.screener.in/company/538706/" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="M17" r:id="rId32" tooltip="https://www.screener.in/company/538706/" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="B18" r:id="rId33" tooltip="https://www.screener.in/company/BCP/" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="M18" r:id="rId34" tooltip="https://www.screener.in/company/BCP/" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="B19" r:id="rId35" tooltip="https://www.screener.in/company/513418/" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="M19" r:id="rId36" tooltip="https://www.screener.in/company/513418/" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="B20" r:id="rId37" tooltip="https://www.screener.in/company/526941/" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="M20" r:id="rId38" tooltip="https://www.screener.in/company/526941/" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="B21" r:id="rId39" tooltip="https://www.screener.in/company/EXXARO/consolidated/" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="M21" r:id="rId40" tooltip="https://www.screener.in/company/EXXARO/consolidated/" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="B22" r:id="rId41" tooltip="https://www.screener.in/company/515085/" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="M22" r:id="rId42" tooltip="https://www.screener.in/company/515085/" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="B23" r:id="rId43" tooltip="https://www.screener.in/company/ELITECON/consolidated/" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="M23" r:id="rId44" tooltip="https://www.screener.in/company/ELITECON/consolidated/" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="B24" r:id="rId45" tooltip="https://www.screener.in/company/SEPC/consolidated/" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="M24" r:id="rId46" tooltip="https://www.screener.in/company/SEPC/consolidated/" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="B25" r:id="rId47" tooltip="https://www.screener.in/company/DBEIL/" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="M25" r:id="rId48" tooltip="https://www.screener.in/company/DBEIL/" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="B26" r:id="rId49" tooltip="https://www.screener.in/company/MADHAVIPL/consolidated/" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="M26" r:id="rId50" tooltip="https://www.screener.in/company/MADHAVIPL/consolidated/" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="B27" r:id="rId51" tooltip="https://www.screener.in/company/TICL/consolidated/" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="M27" r:id="rId52" tooltip="https://www.screener.in/company/TICL/consolidated/" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="B28" r:id="rId53" tooltip="https://www.screener.in/company/SADBHAV/consolidated/" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="M28" r:id="rId54" tooltip="https://www.screener.in/company/SADBHAV/consolidated/" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="B29" r:id="rId55" tooltip="https://www.screener.in/company/NAVKARURB/" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="M29" r:id="rId56" tooltip="https://www.screener.in/company/NAVKARURB/" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="B30" r:id="rId57" tooltip="https://www.screener.in/company/513579/" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="M30" r:id="rId58" tooltip="https://www.screener.in/company/513579/" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="B31" r:id="rId59" tooltip="https://www.screener.in/company/SADHNANIQ/consolidated/" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="M31" r:id="rId60" tooltip="https://www.screener.in/company/SADHNANIQ/consolidated/" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="B32" r:id="rId61" tooltip="https://www.screener.in/company/514440/" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="M32" r:id="rId62" tooltip="https://www.screener.in/company/514440/" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="B33" r:id="rId63" tooltip="https://www.screener.in/company/524564/" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="M33" r:id="rId64" tooltip="https://www.screener.in/company/524564/" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="B34" r:id="rId65" tooltip="https://www.screener.in/company/EMPOWER/consolidated/" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="M34" r:id="rId66" tooltip="https://www.screener.in/company/EMPOWER/consolidated/" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="B35" r:id="rId67" tooltip="https://www.screener.in/company/GVPTECH/" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="M35" r:id="rId68" tooltip="https://www.screener.in/company/GVPTECH/" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="B36" r:id="rId69" tooltip="https://www.screener.in/company/517393/" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="M36" r:id="rId70" tooltip="https://www.screener.in/company/517393/" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="B37" r:id="rId71" tooltip="https://www.screener.in/company/CEREBRAINT/consolidated/" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="M37" r:id="rId72" tooltip="https://www.screener.in/company/CEREBRAINT/consolidated/" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="B38" r:id="rId73" tooltip="https://www.screener.in/company/517356/" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="M38" r:id="rId74" tooltip="https://www.screener.in/company/517356/" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="B39" r:id="rId75" tooltip="https://www.screener.in/company/512175/" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="M39" r:id="rId76" tooltip="https://www.screener.in/company/512175/" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="B40" r:id="rId77" tooltip="https://www.screener.in/company/511716/" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="M40" r:id="rId78" tooltip="https://www.screener.in/company/511716/" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="B41" r:id="rId79" tooltip="https://www.screener.in/company/539149/consolidated/" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="M41" r:id="rId80" tooltip="https://www.screener.in/company/539149/consolidated/" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="B42" r:id="rId81" tooltip="https://www.screener.in/company/503641/consolidated/" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="M42" r:id="rId82" tooltip="https://www.screener.in/company/503641/consolidated/" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="B43" r:id="rId83" tooltip="https://www.screener.in/company/517399/" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="M43" r:id="rId84" tooltip="https://www.screener.in/company/517399/" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="B44" r:id="rId85" tooltip="https://www.screener.in/company/543546/consolidated/" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="M44" r:id="rId86" tooltip="https://www.screener.in/company/543546/consolidated/" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="B45" r:id="rId87" tooltip="https://www.screener.in/company/540955/" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="M45" r:id="rId88" tooltip="https://www.screener.in/company/540955/" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="B46" r:id="rId89" tooltip="https://www.screener.in/company/BTML/consolidated/" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="M46" r:id="rId90" tooltip="https://www.screener.in/company/BTML/consolidated/" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="B47" r:id="rId91" tooltip="https://www.screener.in/company/539519/consolidated/" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="M47" r:id="rId92" tooltip="https://www.screener.in/company/539519/consolidated/" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="B48" r:id="rId93" tooltip="https://www.screener.in/company/539673/" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="M48" r:id="rId94" tooltip="https://www.screener.in/company/539673/" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="B49" r:id="rId95" tooltip="https://www.screener.in/company/542802/consolidated/" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="M49" r:id="rId96" tooltip="https://www.screener.in/company/542802/consolidated/" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="B50" r:id="rId97" tooltip="https://www.screener.in/company/512257/" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="M50" r:id="rId98" tooltip="https://www.screener.in/company/512257/" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="B51" r:id="rId99" tooltip="https://www.screener.in/company/511463/" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="M51" r:id="rId100" tooltip="https://www.screener.in/company/511463/" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="B52" r:id="rId101" tooltip="https://www.screener.in/company/526935/" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="M52" r:id="rId102" tooltip="https://www.screener.in/company/526935/" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="B53" r:id="rId103" tooltip="https://www.screener.in/company/ALANKIT/consolidated/" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="M53" r:id="rId104" tooltip="https://www.screener.in/company/ALANKIT/consolidated/" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="B54" r:id="rId105" tooltip="https://www.screener.in/company/511557/" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="M54" r:id="rId106" tooltip="https://www.screener.in/company/511557/" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="B55" r:id="rId107" tooltip="https://www.screener.in/company/RUCHINFRA/consolidated/" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="M55" r:id="rId108" tooltip="https://www.screener.in/company/RUCHINFRA/consolidated/" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="B56" r:id="rId109" tooltip="https://www.screener.in/company/DAVANGERE/" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="M56" r:id="rId110" tooltip="https://www.screener.in/company/DAVANGERE/" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="B57" r:id="rId111" tooltip="https://www.screener.in/company/OSIAHYPER/" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="M57" r:id="rId112" tooltip="https://www.screener.in/company/OSIAHYPER/" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="B58" r:id="rId113" tooltip="https://www.screener.in/company/FLFL/consolidated/" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="M58" r:id="rId114" tooltip="https://www.screener.in/company/FLFL/consolidated/" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="B59" r:id="rId115" tooltip="https://www.screener.in/company/FEL/" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="M59" r:id="rId116" tooltip="https://www.screener.in/company/FEL/" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="B60" r:id="rId117" tooltip="https://www.screener.in/company/534708/" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="M60" r:id="rId118" tooltip="https://www.screener.in/company/534708/" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="B61" r:id="rId119" tooltip="https://www.screener.in/company/FELDVR/" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="M61" r:id="rId120" tooltip="https://www.screener.in/company/FELDVR/" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="B62" r:id="rId121" tooltip="https://www.screener.in/company/YCCL/consolidated/" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="M62" r:id="rId122" tooltip="https://www.screener.in/company/YCCL/consolidated/" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="B63" r:id="rId123" tooltip="https://www.screener.in/company/UMESLTD/consolidated/" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="M63" r:id="rId124" tooltip="https://www.screener.in/company/UMESLTD/consolidated/" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
+    <hyperlink ref="B64" r:id="rId125" tooltip="https://www.screener.in/company/541865/" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="M64" r:id="rId126" tooltip="https://www.screener.in/company/541865/" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
+    <hyperlink ref="B65" r:id="rId127" tooltip="https://www.screener.in/company/CBAZAAR/consolidated/" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="M65" r:id="rId128" tooltip="https://www.screener.in/company/CBAZAAR/consolidated/" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
+    <hyperlink ref="B66" r:id="rId129" tooltip="https://www.screener.in/company/543521/" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="M66" r:id="rId130" tooltip="https://www.screener.in/company/543521/" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="B67" r:id="rId131" tooltip="https://www.screener.in/company/MKPL/" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
+    <hyperlink ref="M67" r:id="rId132" tooltip="https://www.screener.in/company/MKPL/" xr:uid="{00000000-0004-0000-0000-000083000000}"/>
+    <hyperlink ref="B68" r:id="rId133" tooltip="https://www.screener.in/company/531153/" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
+    <hyperlink ref="M68" r:id="rId134" tooltip="https://www.screener.in/company/531153/" xr:uid="{00000000-0004-0000-0000-000085000000}"/>
+    <hyperlink ref="B69" r:id="rId135" tooltip="https://www.screener.in/company/ZEELEARN/consolidated/" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
+    <hyperlink ref="M69" r:id="rId136" tooltip="https://www.screener.in/company/ZEELEARN/consolidated/" xr:uid="{00000000-0004-0000-0000-000087000000}"/>
+    <hyperlink ref="B70" r:id="rId137" tooltip="https://www.screener.in/company/LCCINFOTEC/" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
+    <hyperlink ref="M70" r:id="rId138" tooltip="https://www.screener.in/company/LCCINFOTEC/" xr:uid="{00000000-0004-0000-0000-000089000000}"/>
+    <hyperlink ref="B71" r:id="rId139" tooltip="https://www.screener.in/company/KEEPLEARN/" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
+    <hyperlink ref="M71" r:id="rId140" tooltip="https://www.screener.in/company/KEEPLEARN/" xr:uid="{00000000-0004-0000-0000-00008B000000}"/>
+    <hyperlink ref="B72" r:id="rId141" tooltip="https://www.screener.in/company/VIRTUALG/consolidated/" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
+    <hyperlink ref="M72" r:id="rId142" tooltip="https://www.screener.in/company/VIRTUALG/consolidated/" xr:uid="{00000000-0004-0000-0000-00008D000000}"/>
+    <hyperlink ref="B73" r:id="rId143" tooltip="https://www.screener.in/company/539761/" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
+    <hyperlink ref="M73" r:id="rId144" tooltip="https://www.screener.in/company/539761/" xr:uid="{00000000-0004-0000-0000-00008F000000}"/>
+    <hyperlink ref="B74" r:id="rId145" tooltip="https://www.screener.in/company/TREEHOUSE/consolidated/" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
+    <hyperlink ref="M74" r:id="rId146" tooltip="https://www.screener.in/company/TREEHOUSE/consolidated/" xr:uid="{00000000-0004-0000-0000-000091000000}"/>
+    <hyperlink ref="B75" r:id="rId147" tooltip="https://www.screener.in/company/MTEDUCARE/consolidated/" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
+    <hyperlink ref="M75" r:id="rId148" tooltip="https://www.screener.in/company/MTEDUCARE/consolidated/" xr:uid="{00000000-0004-0000-0000-000093000000}"/>
+    <hyperlink ref="B76" r:id="rId149" tooltip="https://www.screener.in/company/SAMBHAAV/consolidated/" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
+    <hyperlink ref="M76" r:id="rId150" tooltip="https://www.screener.in/company/SAMBHAAV/consolidated/" xr:uid="{00000000-0004-0000-0000-000095000000}"/>
+    <hyperlink ref="B77" r:id="rId151" tooltip="https://www.screener.in/company/DNAMEDIA/" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
+    <hyperlink ref="M77" r:id="rId152" tooltip="https://www.screener.in/company/DNAMEDIA/" xr:uid="{00000000-0004-0000-0000-000097000000}"/>
+    <hyperlink ref="B78" r:id="rId153" tooltip="https://www.screener.in/company/SHYAMCENT/" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
+    <hyperlink ref="M78" r:id="rId154" tooltip="https://www.screener.in/company/SHYAMCENT/" xr:uid="{00000000-0004-0000-0000-000099000000}"/>
+    <hyperlink ref="B79" r:id="rId155" tooltip="https://www.screener.in/company/532656/consolidated/" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
+    <hyperlink ref="M79" r:id="rId156" tooltip="https://www.screener.in/company/532656/consolidated/" xr:uid="{00000000-0004-0000-0000-00009B000000}"/>
+    <hyperlink ref="B80" r:id="rId157" tooltip="https://www.screener.in/company/IMPEXFERRO/" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
+    <hyperlink ref="M80" r:id="rId158" tooltip="https://www.screener.in/company/IMPEXFERRO/" xr:uid="{00000000-0004-0000-0000-00009D000000}"/>
+    <hyperlink ref="B81" r:id="rId159" tooltip="https://www.screener.in/company/NAGAFERT/consolidated/" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
+    <hyperlink ref="M81" r:id="rId160" tooltip="https://www.screener.in/company/NAGAFERT/consolidated/" xr:uid="{00000000-0004-0000-0000-00009F000000}"/>
+    <hyperlink ref="B82" r:id="rId161" tooltip="https://www.screener.in/company/523277/consolidated/" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
+    <hyperlink ref="M82" r:id="rId162" tooltip="https://www.screener.in/company/523277/consolidated/" xr:uid="{00000000-0004-0000-0000-0000A1000000}"/>
+    <hyperlink ref="B83" r:id="rId163" tooltip="https://www.screener.in/company/532355/consolidated/" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
+    <hyperlink ref="M83" r:id="rId164" tooltip="https://www.screener.in/company/532355/consolidated/" xr:uid="{00000000-0004-0000-0000-0000A3000000}"/>
+    <hyperlink ref="B84" r:id="rId165" tooltip="https://www.screener.in/company/511092/" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
+    <hyperlink ref="M84" r:id="rId166" tooltip="https://www.screener.in/company/511092/" xr:uid="{00000000-0004-0000-0000-0000A5000000}"/>
+    <hyperlink ref="B85" r:id="rId167" tooltip="https://www.screener.in/company/511246/" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
+    <hyperlink ref="M85" r:id="rId168" tooltip="https://www.screener.in/company/511246/" xr:uid="{00000000-0004-0000-0000-0000A7000000}"/>
+    <hyperlink ref="B86" r:id="rId169" tooltip="https://www.screener.in/company/531512/" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
+    <hyperlink ref="M86" r:id="rId170" tooltip="https://www.screener.in/company/531512/" xr:uid="{00000000-0004-0000-0000-0000A9000000}"/>
+    <hyperlink ref="B87" r:id="rId171" tooltip="https://www.screener.in/company/532072/" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
+    <hyperlink ref="M87" r:id="rId172" tooltip="https://www.screener.in/company/532072/" xr:uid="{00000000-0004-0000-0000-0000AB000000}"/>
+    <hyperlink ref="B88" r:id="rId173" tooltip="https://www.screener.in/company/PPSL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
+    <hyperlink ref="M88" r:id="rId174" tooltip="https://www.screener.in/company/PPSL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000AD000000}"/>
+    <hyperlink ref="B89" r:id="rId175" tooltip="https://www.screener.in/company/532160/" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
+    <hyperlink ref="M89" r:id="rId176" tooltip="https://www.screener.in/company/532160/" xr:uid="{00000000-0004-0000-0000-0000AF000000}"/>
+    <hyperlink ref="B90" r:id="rId177" tooltip="https://www.screener.in/company/MOS/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B0000000}"/>
+    <hyperlink ref="M90" r:id="rId178" tooltip="https://www.screener.in/company/MOS/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B1000000}"/>
+    <hyperlink ref="B91" r:id="rId179" tooltip="https://www.screener.in/company/SUVIDHAA/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B2000000}"/>
+    <hyperlink ref="M91" r:id="rId180" tooltip="https://www.screener.in/company/SUVIDHAA/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B3000000}"/>
+    <hyperlink ref="B92" r:id="rId181" tooltip="https://www.screener.in/company/AGSTRA/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B4000000}"/>
+    <hyperlink ref="M92" r:id="rId182" tooltip="https://www.screener.in/company/AGSTRA/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B5000000}"/>
+    <hyperlink ref="B93" r:id="rId183" tooltip="https://www.screener.in/company/526490/" xr:uid="{00000000-0004-0000-0000-0000B6000000}"/>
+    <hyperlink ref="M93" r:id="rId184" tooltip="https://www.screener.in/company/526490/" xr:uid="{00000000-0004-0000-0000-0000B7000000}"/>
+    <hyperlink ref="B94" r:id="rId185" tooltip="https://www.screener.in/company/516062/" xr:uid="{00000000-0004-0000-0000-0000B8000000}"/>
+    <hyperlink ref="M94" r:id="rId186" tooltip="https://www.screener.in/company/516062/" xr:uid="{00000000-0004-0000-0000-0000B9000000}"/>
+    <hyperlink ref="B95" r:id="rId187" tooltip="https://www.screener.in/company/HARDWYN/" xr:uid="{00000000-0004-0000-0000-0000BA000000}"/>
+    <hyperlink ref="M95" r:id="rId188" tooltip="https://www.screener.in/company/HARDWYN/" xr:uid="{00000000-0004-0000-0000-0000BB000000}"/>
+    <hyperlink ref="B96" r:id="rId189" tooltip="https://www.screener.in/company/544188/" xr:uid="{00000000-0004-0000-0000-0000BC000000}"/>
+    <hyperlink ref="M96" r:id="rId190" tooltip="https://www.screener.in/company/544188/" xr:uid="{00000000-0004-0000-0000-0000BD000000}"/>
+    <hyperlink ref="B97" r:id="rId191" tooltip="https://www.screener.in/company/FILATFASH/consolidated/" xr:uid="{00000000-0004-0000-0000-0000BE000000}"/>
+    <hyperlink ref="M97" r:id="rId192" tooltip="https://www.screener.in/company/FILATFASH/consolidated/" xr:uid="{00000000-0004-0000-0000-0000BF000000}"/>
+    <hyperlink ref="B98" r:id="rId193" tooltip="https://www.screener.in/company/LAL/" xr:uid="{00000000-0004-0000-0000-0000C0000000}"/>
+    <hyperlink ref="M98" r:id="rId194" tooltip="https://www.screener.in/company/LAL/" xr:uid="{00000000-0004-0000-0000-0000C1000000}"/>
+    <hyperlink ref="B99" r:id="rId195" tooltip="https://www.screener.in/company/539216/consolidated/" xr:uid="{00000000-0004-0000-0000-0000C2000000}"/>
+    <hyperlink ref="M99" r:id="rId196" tooltip="https://www.screener.in/company/539216/consolidated/" xr:uid="{00000000-0004-0000-0000-0000C3000000}"/>
+    <hyperlink ref="B100" r:id="rId197" tooltip="https://www.screener.in/company/VINNY/" xr:uid="{00000000-0004-0000-0000-0000C4000000}"/>
+    <hyperlink ref="M100" r:id="rId198" tooltip="https://www.screener.in/company/VINNY/" xr:uid="{00000000-0004-0000-0000-0000C5000000}"/>
+    <hyperlink ref="B101" r:id="rId199" tooltip="https://www.screener.in/company/CELEBRITY/" xr:uid="{00000000-0004-0000-0000-0000C6000000}"/>
+    <hyperlink ref="M101" r:id="rId200" tooltip="https://www.screener.in/company/CELEBRITY/" xr:uid="{00000000-0004-0000-0000-0000C7000000}"/>
+    <hyperlink ref="B102" r:id="rId201" tooltip="https://www.screener.in/company/542579/" xr:uid="{00000000-0004-0000-0000-0000C8000000}"/>
+    <hyperlink ref="M102" r:id="rId202" tooltip="https://www.screener.in/company/542579/" xr:uid="{00000000-0004-0000-0000-0000C9000000}"/>
+    <hyperlink ref="B103" r:id="rId203" tooltip="https://www.screener.in/company/540252/" xr:uid="{00000000-0004-0000-0000-0000CA000000}"/>
+    <hyperlink ref="M103" r:id="rId204" tooltip="https://www.screener.in/company/540252/" xr:uid="{00000000-0004-0000-0000-0000CB000000}"/>
+    <hyperlink ref="B104" r:id="rId205" tooltip="https://www.screener.in/company/523373/consolidated/" xr:uid="{00000000-0004-0000-0000-0000CC000000}"/>
+    <hyperlink ref="M104" r:id="rId206" tooltip="https://www.screener.in/company/523373/consolidated/" xr:uid="{00000000-0004-0000-0000-0000CD000000}"/>
+    <hyperlink ref="B105" r:id="rId207" tooltip="https://www.screener.in/company/MOKSH/" xr:uid="{00000000-0004-0000-0000-0000CE000000}"/>
+    <hyperlink ref="M105" r:id="rId208" tooltip="https://www.screener.in/company/MOKSH/" xr:uid="{00000000-0004-0000-0000-0000CF000000}"/>
+    <hyperlink ref="B106" r:id="rId209" tooltip="https://www.screener.in/company/512047/" xr:uid="{00000000-0004-0000-0000-0000D0000000}"/>
+    <hyperlink ref="M106" r:id="rId210" tooltip="https://www.screener.in/company/512047/" xr:uid="{00000000-0004-0000-0000-0000D1000000}"/>
+    <hyperlink ref="B107" r:id="rId211" tooltip="https://www.screener.in/company/523387/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D2000000}"/>
+    <hyperlink ref="M107" r:id="rId212" tooltip="https://www.screener.in/company/523387/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D3000000}"/>
+    <hyperlink ref="B108" r:id="rId213" tooltip="https://www.screener.in/company/530525/" xr:uid="{00000000-0004-0000-0000-0000D4000000}"/>
+    <hyperlink ref="M108" r:id="rId214" tooltip="https://www.screener.in/company/530525/" xr:uid="{00000000-0004-0000-0000-0000D5000000}"/>
+    <hyperlink ref="B109" r:id="rId215" tooltip="https://www.screener.in/company/531626/" xr:uid="{00000000-0004-0000-0000-0000D6000000}"/>
+    <hyperlink ref="M109" r:id="rId216" tooltip="https://www.screener.in/company/531626/" xr:uid="{00000000-0004-0000-0000-0000D7000000}"/>
+    <hyperlink ref="B110" r:id="rId217" tooltip="https://www.screener.in/company/KANANIIND/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D8000000}"/>
+    <hyperlink ref="M110" r:id="rId218" tooltip="https://www.screener.in/company/KANANIIND/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D9000000}"/>
+    <hyperlink ref="B111" r:id="rId219" tooltip="https://www.screener.in/company/540953/" xr:uid="{00000000-0004-0000-0000-0000DA000000}"/>
+    <hyperlink ref="M111" r:id="rId220" tooltip="https://www.screener.in/company/540953/" xr:uid="{00000000-0004-0000-0000-0000DB000000}"/>
+    <hyperlink ref="B112" r:id="rId221" tooltip="https://www.screener.in/company/ORIENTALTL/" xr:uid="{00000000-0004-0000-0000-0000DC000000}"/>
+    <hyperlink ref="M112" r:id="rId222" tooltip="https://www.screener.in/company/ORIENTALTL/" xr:uid="{00000000-0004-0000-0000-0000DD000000}"/>
+    <hyperlink ref="B113" r:id="rId223" tooltip="https://www.screener.in/company/JYOTISTRUC/consolidated/" xr:uid="{00000000-0004-0000-0000-0000DE000000}"/>
+    <hyperlink ref="M113" r:id="rId224" tooltip="https://www.screener.in/company/JYOTISTRUC/consolidated/" xr:uid="{00000000-0004-0000-0000-0000DF000000}"/>
+    <hyperlink ref="B114" r:id="rId225" tooltip="https://www.screener.in/company/BILVYAPAR/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E0000000}"/>
+    <hyperlink ref="M114" r:id="rId226" tooltip="https://www.screener.in/company/BILVYAPAR/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E1000000}"/>
+    <hyperlink ref="B115" r:id="rId227" tooltip="https://www.screener.in/company/531658/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E2000000}"/>
+    <hyperlink ref="M115" r:id="rId228" tooltip="https://www.screener.in/company/531658/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E3000000}"/>
+    <hyperlink ref="B116" r:id="rId229" tooltip="https://www.screener.in/company/HLVLTD/" xr:uid="{00000000-0004-0000-0000-0000E4000000}"/>
+    <hyperlink ref="M116" r:id="rId230" tooltip="https://www.screener.in/company/HLVLTD/" xr:uid="{00000000-0004-0000-0000-0000E5000000}"/>
+    <hyperlink ref="B117" r:id="rId231" tooltip="https://www.screener.in/company/531663/" xr:uid="{00000000-0004-0000-0000-0000E6000000}"/>
+    <hyperlink ref="M117" r:id="rId232" tooltip="https://www.screener.in/company/531663/" xr:uid="{00000000-0004-0000-0000-0000E7000000}"/>
+    <hyperlink ref="B118" r:id="rId233" tooltip="https://www.screener.in/company/RHFL/" xr:uid="{00000000-0004-0000-0000-0000E8000000}"/>
+    <hyperlink ref="M118" r:id="rId234" tooltip="https://www.screener.in/company/RHFL/" xr:uid="{00000000-0004-0000-0000-0000E9000000}"/>
+    <hyperlink ref="B119" r:id="rId235" tooltip="https://www.screener.in/company/539017/" xr:uid="{00000000-0004-0000-0000-0000EA000000}"/>
+    <hyperlink ref="M119" r:id="rId236" tooltip="https://www.screener.in/company/539017/" xr:uid="{00000000-0004-0000-0000-0000EB000000}"/>
+    <hyperlink ref="B120" r:id="rId237" tooltip="https://www.screener.in/company/SALASAR/consolidated/" xr:uid="{00000000-0004-0000-0000-0000EC000000}"/>
+    <hyperlink ref="M120" r:id="rId238" tooltip="https://www.screener.in/company/SALASAR/consolidated/" xr:uid="{00000000-0004-0000-0000-0000ED000000}"/>
+    <hyperlink ref="B121" r:id="rId239" tooltip="https://www.screener.in/company/DPSCLTD/consolidated/" xr:uid="{00000000-0004-0000-0000-0000EE000000}"/>
+    <hyperlink ref="M121" r:id="rId240" tooltip="https://www.screener.in/company/DPSCLTD/consolidated/" xr:uid="{00000000-0004-0000-0000-0000EF000000}"/>
+    <hyperlink ref="B122" r:id="rId241" tooltip="https://www.screener.in/company/538765/" xr:uid="{00000000-0004-0000-0000-0000F0000000}"/>
+    <hyperlink ref="M122" r:id="rId242" tooltip="https://www.screener.in/company/538765/" xr:uid="{00000000-0004-0000-0000-0000F1000000}"/>
+    <hyperlink ref="B123" r:id="rId243" tooltip="https://www.screener.in/company/503663/" xr:uid="{00000000-0004-0000-0000-0000F2000000}"/>
+    <hyperlink ref="M123" r:id="rId244" tooltip="https://www.screener.in/company/503663/" xr:uid="{00000000-0004-0000-0000-0000F3000000}"/>
+    <hyperlink ref="B124" r:id="rId245" tooltip="https://www.screener.in/company/538451/" xr:uid="{00000000-0004-0000-0000-0000F4000000}"/>
+    <hyperlink ref="M124" r:id="rId246" tooltip="https://www.screener.in/company/538451/" xr:uid="{00000000-0004-0000-0000-0000F5000000}"/>
+    <hyperlink ref="B125" r:id="rId247" tooltip="https://www.screener.in/company/509051/" xr:uid="{00000000-0004-0000-0000-0000F6000000}"/>
+    <hyperlink ref="M125" r:id="rId248" tooltip="https://www.screener.in/company/509051/" xr:uid="{00000000-0004-0000-0000-0000F7000000}"/>
+    <hyperlink ref="B126" r:id="rId249" tooltip="https://www.screener.in/company/PARASPETRO/" xr:uid="{00000000-0004-0000-0000-0000F8000000}"/>
+    <hyperlink ref="M126" r:id="rId250" tooltip="https://www.screener.in/company/PARASPETRO/" xr:uid="{00000000-0004-0000-0000-0000F9000000}"/>
+    <hyperlink ref="B127" r:id="rId251" tooltip="https://www.screener.in/company/509053/consolidated/" xr:uid="{00000000-0004-0000-0000-0000FA000000}"/>
+    <hyperlink ref="M127" r:id="rId252" tooltip="https://www.screener.in/company/509053/consolidated/" xr:uid="{00000000-0004-0000-0000-0000FB000000}"/>
+    <hyperlink ref="B128" r:id="rId253" tooltip="https://www.screener.in/company/539091/" xr:uid="{00000000-0004-0000-0000-0000FC000000}"/>
+    <hyperlink ref="M128" r:id="rId254" tooltip="https://www.screener.in/company/539091/" xr:uid="{00000000-0004-0000-0000-0000FD000000}"/>
+    <hyperlink ref="B129" r:id="rId255" tooltip="https://www.screener.in/company/ANKITMETAL/" xr:uid="{00000000-0004-0000-0000-0000FE000000}"/>
+    <hyperlink ref="M129" r:id="rId256" tooltip="https://www.screener.in/company/ANKITMETAL/" xr:uid="{00000000-0004-0000-0000-0000FF000000}"/>
+    <hyperlink ref="B130" r:id="rId257" tooltip="https://www.screener.in/company/RAMASTEEL/consolidated/" xr:uid="{00000000-0004-0000-0000-000000010000}"/>
+    <hyperlink ref="M130" r:id="rId258" tooltip="https://www.screener.in/company/RAMASTEEL/consolidated/" xr:uid="{00000000-0004-0000-0000-000001010000}"/>
+    <hyperlink ref="B131" r:id="rId259" tooltip="https://www.screener.in/company/SHAH/consolidated/" xr:uid="{00000000-0004-0000-0000-000002010000}"/>
+    <hyperlink ref="M131" r:id="rId260" tooltip="https://www.screener.in/company/SHAH/consolidated/" xr:uid="{00000000-0004-0000-0000-000003010000}"/>
+    <hyperlink ref="B132" r:id="rId261" tooltip="https://www.screener.in/company/KRITIKA/" xr:uid="{00000000-0004-0000-0000-000004010000}"/>
+    <hyperlink ref="M132" r:id="rId262" tooltip="https://www.screener.in/company/KRITIKA/" xr:uid="{00000000-0004-0000-0000-000005010000}"/>
+    <hyperlink ref="B133" r:id="rId263" tooltip="https://www.screener.in/company/534064/" xr:uid="{00000000-0004-0000-0000-000006010000}"/>
+    <hyperlink ref="M133" r:id="rId264" tooltip="https://www.screener.in/company/534064/" xr:uid="{00000000-0004-0000-0000-000007010000}"/>
+    <hyperlink ref="B134" r:id="rId265" tooltip="https://www.screener.in/company/SUPREMEENG/" xr:uid="{00000000-0004-0000-0000-000008010000}"/>
+    <hyperlink ref="M134" r:id="rId266" tooltip="https://www.screener.in/company/SUPREMEENG/" xr:uid="{00000000-0004-0000-0000-000009010000}"/>
+    <hyperlink ref="B135" r:id="rId267" tooltip="https://www.screener.in/company/ZENITHSTL/consolidated/" xr:uid="{00000000-0004-0000-0000-00000A010000}"/>
+    <hyperlink ref="M135" r:id="rId268" tooltip="https://www.screener.in/company/ZENITHSTL/consolidated/" xr:uid="{00000000-0004-0000-0000-00000B010000}"/>
+    <hyperlink ref="B136" r:id="rId269" tooltip="https://www.screener.in/company/PRAKASHSTL/" xr:uid="{00000000-0004-0000-0000-00000C010000}"/>
+    <hyperlink ref="M136" r:id="rId270" tooltip="https://www.screener.in/company/PRAKASHSTL/" xr:uid="{00000000-0004-0000-0000-00000D010000}"/>
+    <hyperlink ref="B137" r:id="rId271" tooltip="https://www.screener.in/company/BCG/consolidated/" xr:uid="{00000000-0004-0000-0000-00000E010000}"/>
+    <hyperlink ref="M137" r:id="rId272" tooltip="https://www.screener.in/company/BCG/consolidated/" xr:uid="{00000000-0004-0000-0000-00000F010000}"/>
+    <hyperlink ref="B138" r:id="rId273" tooltip="https://www.screener.in/company/534535/consolidated/" xr:uid="{00000000-0004-0000-0000-000010010000}"/>
+    <hyperlink ref="M138" r:id="rId274" tooltip="https://www.screener.in/company/534535/consolidated/" xr:uid="{00000000-0004-0000-0000-000011010000}"/>
+    <hyperlink ref="B139" r:id="rId275" tooltip="https://www.screener.in/company/VAKRANGEE/consolidated/" xr:uid="{00000000-0004-0000-0000-000012010000}"/>
+    <hyperlink ref="M139" r:id="rId276" tooltip="https://www.screener.in/company/VAKRANGEE/consolidated/" xr:uid="{00000000-0004-0000-0000-000013010000}"/>
+    <hyperlink ref="B140" r:id="rId277" tooltip="https://www.screener.in/company/FCSSOFT/consolidated/" xr:uid="{00000000-0004-0000-0000-000014010000}"/>
+    <hyperlink ref="M140" r:id="rId278" tooltip="https://www.screener.in/company/FCSSOFT/consolidated/" xr:uid="{00000000-0004-0000-0000-000015010000}"/>
+    <hyperlink ref="B141" r:id="rId279" tooltip="https://www.screener.in/company/ASMS/consolidated/" xr:uid="{00000000-0004-0000-0000-000016010000}"/>
+    <hyperlink ref="M141" r:id="rId280" tooltip="https://www.screener.in/company/ASMS/consolidated/" xr:uid="{00000000-0004-0000-0000-000017010000}"/>
+    <hyperlink ref="B142" r:id="rId281" tooltip="https://www.screener.in/company/VLEGOV/" xr:uid="{00000000-0004-0000-0000-000018010000}"/>
+    <hyperlink ref="M142" r:id="rId282" tooltip="https://www.screener.in/company/VLEGOV/" xr:uid="{00000000-0004-0000-0000-000019010000}"/>
+    <hyperlink ref="B143" r:id="rId283" tooltip="https://www.screener.in/company/521005/" xr:uid="{00000000-0004-0000-0000-00001A010000}"/>
+    <hyperlink ref="M143" r:id="rId284" tooltip="https://www.screener.in/company/521005/" xr:uid="{00000000-0004-0000-0000-00001B010000}"/>
+    <hyperlink ref="B144" r:id="rId285" tooltip="https://www.screener.in/company/CRSL/" xr:uid="{00000000-0004-0000-0000-00001C010000}"/>
+    <hyperlink ref="M144" r:id="rId286" tooltip="https://www.screener.in/company/CRSL/" xr:uid="{00000000-0004-0000-0000-00001D010000}"/>
+    <hyperlink ref="B145" r:id="rId287" tooltip="https://www.screener.in/company/SGLRES/" xr:uid="{00000000-0004-0000-0000-00001E010000}"/>
+    <hyperlink ref="M145" r:id="rId288" tooltip="https://www.screener.in/company/SGLRES/" xr:uid="{00000000-0004-0000-0000-00001F010000}"/>
+    <hyperlink ref="B146" r:id="rId289" tooltip="https://www.screener.in/company/SUPTANERY/consolidated/" xr:uid="{00000000-0004-0000-0000-000020010000}"/>
+    <hyperlink ref="M146" r:id="rId290" tooltip="https://www.screener.in/company/SUPTANERY/consolidated/" xr:uid="{00000000-0004-0000-0000-000021010000}"/>
+    <hyperlink ref="B147" r:id="rId291" tooltip="https://www.screener.in/company/AKI/consolidated/" xr:uid="{00000000-0004-0000-0000-000022010000}"/>
+    <hyperlink ref="M147" r:id="rId292" tooltip="https://www.screener.in/company/AKI/consolidated/" xr:uid="{00000000-0004-0000-0000-000023010000}"/>
+    <hyperlink ref="B148" r:id="rId293" tooltip="https://www.screener.in/company/541771/" xr:uid="{00000000-0004-0000-0000-000024010000}"/>
+    <hyperlink ref="M148" r:id="rId294" tooltip="https://www.screener.in/company/541771/" xr:uid="{00000000-0004-0000-0000-000025010000}"/>
+    <hyperlink ref="B149" r:id="rId295" tooltip="https://www.screener.in/company/523242/" xr:uid="{00000000-0004-0000-0000-000026010000}"/>
+    <hyperlink ref="M149" r:id="rId296" tooltip="https://www.screener.in/company/523242/" xr:uid="{00000000-0004-0000-0000-000027010000}"/>
+    <hyperlink ref="B150" r:id="rId297" tooltip="https://www.screener.in/company/526415/consolidated/" xr:uid="{00000000-0004-0000-0000-000028010000}"/>
+    <hyperlink ref="M150" r:id="rId298" tooltip="https://www.screener.in/company/526415/consolidated/" xr:uid="{00000000-0004-0000-0000-000029010000}"/>
+    <hyperlink ref="B151" r:id="rId299" tooltip="https://www.screener.in/company/534190/" xr:uid="{00000000-0004-0000-0000-00002A010000}"/>
+    <hyperlink ref="M151" r:id="rId300" tooltip="https://www.screener.in/company/534190/" xr:uid="{00000000-0004-0000-0000-00002B010000}"/>
+    <hyperlink ref="B152" r:id="rId301" tooltip="https://www.screener.in/company/531977/" xr:uid="{00000000-0004-0000-0000-00002C010000}"/>
+    <hyperlink ref="M152" r:id="rId302" tooltip="https://www.screener.in/company/531977/" xr:uid="{00000000-0004-0000-0000-00002D010000}"/>
+    <hyperlink ref="B153" r:id="rId303" tooltip="https://www.screener.in/company/RADIOCITY/" xr:uid="{00000000-0004-0000-0000-00002E010000}"/>
+    <hyperlink ref="M153" r:id="rId304" tooltip="https://www.screener.in/company/RADIOCITY/" xr:uid="{00000000-0004-0000-0000-00002F010000}"/>
+    <hyperlink ref="B154" r:id="rId305" tooltip="https://www.screener.in/company/539175/" xr:uid="{00000000-0004-0000-0000-000030010000}"/>
+    <hyperlink ref="M154" r:id="rId306" tooltip="https://www.screener.in/company/539175/" xr:uid="{00000000-0004-0000-0000-000031010000}"/>
+    <hyperlink ref="B155" r:id="rId307" tooltip="https://www.screener.in/company/STUDIOLSD/" xr:uid="{00000000-0004-0000-0000-000032010000}"/>
+    <hyperlink ref="M155" r:id="rId308" tooltip="https://www.screener.in/company/STUDIOLSD/" xr:uid="{00000000-0004-0000-0000-000033010000}"/>
+    <hyperlink ref="B156" r:id="rId309" tooltip="https://www.screener.in/company/NEXTMEDIA/" xr:uid="{00000000-0004-0000-0000-000034010000}"/>
+    <hyperlink ref="M156" r:id="rId310" tooltip="https://www.screener.in/company/NEXTMEDIA/" xr:uid="{00000000-0004-0000-0000-000035010000}"/>
+    <hyperlink ref="B157" r:id="rId311" tooltip="https://www.screener.in/company/512499/" xr:uid="{00000000-0004-0000-0000-000036010000}"/>
+    <hyperlink ref="M157" r:id="rId312" tooltip="https://www.screener.in/company/512499/" xr:uid="{00000000-0004-0000-0000-000037010000}"/>
+    <hyperlink ref="B158" r:id="rId313" tooltip="https://www.screener.in/company/RADAAN/consolidated/" xr:uid="{00000000-0004-0000-0000-000038010000}"/>
+    <hyperlink ref="M158" r:id="rId314" tooltip="https://www.screener.in/company/RADAAN/consolidated/" xr:uid="{00000000-0004-0000-0000-000039010000}"/>
+    <hyperlink ref="B159" r:id="rId315" tooltip="https://www.screener.in/company/INSPIRE/" xr:uid="{00000000-0004-0000-0000-00003A010000}"/>
+    <hyperlink ref="M159" r:id="rId316" tooltip="https://www.screener.in/company/INSPIRE/" xr:uid="{00000000-0004-0000-0000-00003B010000}"/>
+    <hyperlink ref="B160" r:id="rId317" tooltip="https://www.screener.in/company/CREATIVEYE/" xr:uid="{00000000-0004-0000-0000-00003C010000}"/>
+    <hyperlink ref="M160" r:id="rId318" tooltip="https://www.screener.in/company/CREATIVEYE/" xr:uid="{00000000-0004-0000-0000-00003D010000}"/>
+    <hyperlink ref="B161" r:id="rId319" tooltip="https://www.screener.in/company/501945/" xr:uid="{00000000-0004-0000-0000-00003E010000}"/>
+    <hyperlink ref="M161" r:id="rId320" tooltip="https://www.screener.in/company/501945/" xr:uid="{00000000-0004-0000-0000-00003F010000}"/>
+    <hyperlink ref="B162" r:id="rId321" tooltip="https://www.screener.in/company/AFIL/" xr:uid="{00000000-0004-0000-0000-000040010000}"/>
+    <hyperlink ref="M162" r:id="rId322" tooltip="https://www.screener.in/company/AFIL/" xr:uid="{00000000-0004-0000-0000-000041010000}"/>
+    <hyperlink ref="B163" r:id="rId323" tooltip="https://www.screener.in/company/532320/consolidated/" xr:uid="{00000000-0004-0000-0000-000042010000}"/>
+    <hyperlink ref="M163" r:id="rId324" tooltip="https://www.screener.in/company/532320/consolidated/" xr:uid="{00000000-0004-0000-0000-000043010000}"/>
+    <hyperlink ref="B164" r:id="rId325" tooltip="https://www.screener.in/company/532275/" xr:uid="{00000000-0004-0000-0000-000044010000}"/>
+    <hyperlink ref="M164" r:id="rId326" tooltip="https://www.screener.in/company/532275/" xr:uid="{00000000-0004-0000-0000-000045010000}"/>
+    <hyperlink ref="B165" r:id="rId327" tooltip="https://www.screener.in/company/526961/consolidated/" xr:uid="{00000000-0004-0000-0000-000046010000}"/>
+    <hyperlink ref="M165" r:id="rId328" tooltip="https://www.screener.in/company/526961/consolidated/" xr:uid="{00000000-0004-0000-0000-000047010000}"/>
+    <hyperlink ref="B166" r:id="rId329" tooltip="https://www.screener.in/company/534060/" xr:uid="{00000000-0004-0000-0000-000048010000}"/>
+    <hyperlink ref="M166" r:id="rId330" tooltip="https://www.screener.in/company/534060/" xr:uid="{00000000-0004-0000-0000-000049010000}"/>
+    <hyperlink ref="B167" r:id="rId331" tooltip="https://www.screener.in/company/507962/" xr:uid="{00000000-0004-0000-0000-00004A010000}"/>
+    <hyperlink ref="M167" r:id="rId332" tooltip="https://www.screener.in/company/507962/" xr:uid="{00000000-0004-0000-0000-00004B010000}"/>
+    <hyperlink ref="B168" r:id="rId333" tooltip="https://www.screener.in/company/530557/" xr:uid="{00000000-0004-0000-0000-00004C010000}"/>
+    <hyperlink ref="M168" r:id="rId334" tooltip="https://www.screener.in/company/530557/" xr:uid="{00000000-0004-0000-0000-00004D010000}"/>
+    <hyperlink ref="B169" r:id="rId335" tooltip="https://www.screener.in/company/538860/" xr:uid="{00000000-0004-0000-0000-00004E010000}"/>
+    <hyperlink ref="M169" r:id="rId336" tooltip="https://www.screener.in/company/538860/" xr:uid="{00000000-0004-0000-0000-00004F010000}"/>
+    <hyperlink ref="B170" r:id="rId337" tooltip="https://www.screener.in/company/AAKASH/" xr:uid="{00000000-0004-0000-0000-000050010000}"/>
+    <hyperlink ref="M170" r:id="rId338" tooltip="https://www.screener.in/company/AAKASH/" xr:uid="{00000000-0004-0000-0000-000051010000}"/>
+    <hyperlink ref="B171" r:id="rId339" tooltip="https://www.screener.in/company/SARVESHWAR/consolidated/" xr:uid="{00000000-0004-0000-0000-000052010000}"/>
+    <hyperlink ref="M171" r:id="rId340" tooltip="https://www.screener.in/company/SARVESHWAR/consolidated/" xr:uid="{00000000-0004-0000-0000-000053010000}"/>
+    <hyperlink ref="B172" r:id="rId341" tooltip="https://www.screener.in/company/526445/consolidated/" xr:uid="{00000000-0004-0000-0000-000054010000}"/>
+    <hyperlink ref="M172" r:id="rId342" tooltip="https://www.screener.in/company/526445/consolidated/" xr:uid="{00000000-0004-0000-0000-000055010000}"/>
+    <hyperlink ref="B173" r:id="rId343" tooltip="https://www.screener.in/company/526899/" xr:uid="{00000000-0004-0000-0000-000056010000}"/>
+    <hyperlink ref="M173" r:id="rId344" tooltip="https://www.screener.in/company/526899/" xr:uid="{00000000-0004-0000-0000-000057010000}"/>
+    <hyperlink ref="B174" r:id="rId345" tooltip="https://www.screener.in/company/523467/" xr:uid="{00000000-0004-0000-0000-000058010000}"/>
+    <hyperlink ref="M174" r:id="rId346" tooltip="https://www.screener.in/company/523467/" xr:uid="{00000000-0004-0000-0000-000059010000}"/>
+    <hyperlink ref="B175" r:id="rId347" tooltip="https://www.screener.in/company/URJA/consolidated/" xr:uid="{00000000-0004-0000-0000-00005A010000}"/>
+    <hyperlink ref="M175" r:id="rId348" tooltip="https://www.screener.in/company/URJA/consolidated/" xr:uid="{00000000-0004-0000-0000-00005B010000}"/>
+    <hyperlink ref="B176" r:id="rId349" tooltip="https://www.screener.in/company/DELPHIFX/consolidated/" xr:uid="{00000000-0004-0000-0000-00005C010000}"/>
+    <hyperlink ref="M176" r:id="rId350" tooltip="https://www.screener.in/company/DELPHIFX/consolidated/" xr:uid="{00000000-0004-0000-0000-00005D010000}"/>
+    <hyperlink ref="B177" r:id="rId351" tooltip="https://www.screener.in/company/GATECH/" xr:uid="{00000000-0004-0000-0000-00005E010000}"/>
+    <hyperlink ref="M177" r:id="rId352" tooltip="https://www.screener.in/company/GATECH/" xr:uid="{00000000-0004-0000-0000-00005F010000}"/>
+    <hyperlink ref="B178" r:id="rId353" tooltip="https://www.screener.in/company/512018/consolidated/" xr:uid="{00000000-0004-0000-0000-000060010000}"/>
+    <hyperlink ref="M178" r:id="rId354" tooltip="https://www.screener.in/company/512018/consolidated/" xr:uid="{00000000-0004-0000-0000-000061010000}"/>
+    <hyperlink ref="B179" r:id="rId355" tooltip="https://www.screener.in/company/530881/" xr:uid="{00000000-0004-0000-0000-000062010000}"/>
+    <hyperlink ref="M179" r:id="rId356" tooltip="https://www.screener.in/company/530881/" xr:uid="{00000000-0004-0000-0000-000063010000}"/>
+    <hyperlink ref="B180" r:id="rId357" tooltip="https://www.screener.in/company/531950/consolidated/" xr:uid="{00000000-0004-0000-0000-000064010000}"/>
+    <hyperlink ref="M180" r:id="rId358" tooltip="https://www.screener.in/company/531950/consolidated/" xr:uid="{00000000-0004-0000-0000-000065010000}"/>
+    <hyperlink ref="B181" r:id="rId359" tooltip="https://www.screener.in/company/539132/" xr:uid="{00000000-0004-0000-0000-000066010000}"/>
+    <hyperlink ref="M181" r:id="rId360" tooltip="https://www.screener.in/company/539132/" xr:uid="{00000000-0004-0000-0000-000067010000}"/>
+    <hyperlink ref="B182" r:id="rId361" tooltip="https://www.screener.in/company/517554/consolidated/" xr:uid="{00000000-0004-0000-0000-000068010000}"/>
+    <hyperlink ref="M182" r:id="rId362" tooltip="https://www.screener.in/company/517554/consolidated/" xr:uid="{00000000-0004-0000-0000-000069010000}"/>
+    <hyperlink ref="B183" r:id="rId363" tooltip="https://www.screener.in/company/524614/" xr:uid="{00000000-0004-0000-0000-00006A010000}"/>
+    <hyperlink ref="M183" r:id="rId364" tooltip="https://www.screener.in/company/524614/" xr:uid="{00000000-0004-0000-0000-00006B010000}"/>
+    <hyperlink ref="B184" r:id="rId365" tooltip="https://www.screener.in/company/SANWARIA/consolidated/" xr:uid="{00000000-0004-0000-0000-00006C010000}"/>
+    <hyperlink ref="M184" r:id="rId366" tooltip="https://www.screener.in/company/SANWARIA/consolidated/" xr:uid="{00000000-0004-0000-0000-00006D010000}"/>
+    <hyperlink ref="B185" r:id="rId367" tooltip="https://www.screener.in/company/531716/" xr:uid="{00000000-0004-0000-0000-00006E010000}"/>
+    <hyperlink ref="M185" r:id="rId368" tooltip="https://www.screener.in/company/531716/" xr:uid="{00000000-0004-0000-0000-00006F010000}"/>
+    <hyperlink ref="B186" r:id="rId369" tooltip="https://www.screener.in/company/539219/consolidated/" xr:uid="{00000000-0004-0000-0000-000070010000}"/>
+    <hyperlink ref="M186" r:id="rId370" tooltip="https://www.screener.in/company/539219/consolidated/" xr:uid="{00000000-0004-0000-0000-000071010000}"/>
+    <hyperlink ref="B187" r:id="rId371" tooltip="https://www.screener.in/company/GTL/" xr:uid="{00000000-0004-0000-0000-000072010000}"/>
+    <hyperlink ref="M187" r:id="rId372" tooltip="https://www.screener.in/company/GTL/" xr:uid="{00000000-0004-0000-0000-000073010000}"/>
+    <hyperlink ref="B188" r:id="rId373" tooltip="https://www.screener.in/company/ALOKINDS/consolidated/" xr:uid="{00000000-0004-0000-0000-000074010000}"/>
+    <hyperlink ref="M188" r:id="rId374" tooltip="https://www.screener.in/company/ALOKINDS/consolidated/" xr:uid="{00000000-0004-0000-0000-000075010000}"/>
+    <hyperlink ref="B189" r:id="rId375" tooltip="https://www.screener.in/company/NDL/" xr:uid="{00000000-0004-0000-0000-000076010000}"/>
+    <hyperlink ref="M189" r:id="rId376" tooltip="https://www.screener.in/company/NDL/" xr:uid="{00000000-0004-0000-0000-000077010000}"/>
+    <hyperlink ref="B190" r:id="rId377" tooltip="https://www.screener.in/company/AXITA/" xr:uid="{00000000-0004-0000-0000-000078010000}"/>
+    <hyperlink ref="M190" r:id="rId378" tooltip="https://www.screener.in/company/AXITA/" xr:uid="{00000000-0004-0000-0000-000079010000}"/>
+    <hyperlink ref="B191" r:id="rId379" tooltip="https://www.screener.in/company/VARDMNPOLY/" xr:uid="{00000000-0004-0000-0000-00007A010000}"/>
+    <hyperlink ref="M191" r:id="rId380" tooltip="https://www.screener.in/company/VARDMNPOLY/" xr:uid="{00000000-0004-0000-0000-00007B010000}"/>
+    <hyperlink ref="B192" r:id="rId381" tooltip="https://www.screener.in/company/RNBDENIMS/consolidated/" xr:uid="{00000000-0004-0000-0000-00007C010000}"/>
+    <hyperlink ref="M192" r:id="rId382" tooltip="https://www.screener.in/company/RNBDENIMS/consolidated/" xr:uid="{00000000-0004-0000-0000-00007D010000}"/>
+    <hyperlink ref="B193" r:id="rId383" tooltip="https://www.screener.in/company/TTL/" xr:uid="{00000000-0004-0000-0000-00007E010000}"/>
+    <hyperlink ref="M193" r:id="rId384" tooltip="https://www.screener.in/company/TTL/" xr:uid="{00000000-0004-0000-0000-00007F010000}"/>
+    <hyperlink ref="B194" r:id="rId385" tooltip="https://www.screener.in/company/531411/" xr:uid="{00000000-0004-0000-0000-000080010000}"/>
+    <hyperlink ref="M194" r:id="rId386" tooltip="https://www.screener.in/company/531411/" xr:uid="{00000000-0004-0000-0000-000081010000}"/>
+    <hyperlink ref="B195" r:id="rId387" tooltip="https://www.screener.in/company/530185/" xr:uid="{00000000-0004-0000-0000-000082010000}"/>
+    <hyperlink ref="M195" r:id="rId388" tooltip="https://www.screener.in/company/530185/" xr:uid="{00000000-0004-0000-0000-000083010000}"/>
+    <hyperlink ref="B196" r:id="rId389" tooltip="https://www.screener.in/company/GLOBE/consolidated/" xr:uid="{00000000-0004-0000-0000-000084010000}"/>
+    <hyperlink ref="M196" r:id="rId390" tooltip="https://www.screener.in/company/GLOBE/consolidated/" xr:uid="{00000000-0004-0000-0000-000085010000}"/>
+    <hyperlink ref="B197" r:id="rId391" tooltip="https://www.screener.in/company/BHANDARI/" xr:uid="{00000000-0004-0000-0000-000086010000}"/>
+    <hyperlink ref="M197" r:id="rId392" tooltip="https://www.screener.in/company/BHANDARI/" xr:uid="{00000000-0004-0000-0000-000087010000}"/>
+    <hyperlink ref="B198" r:id="rId393" tooltip="https://www.screener.in/company/539594/consolidated/" xr:uid="{00000000-0004-0000-0000-000088010000}"/>
+    <hyperlink ref="M198" r:id="rId394" tooltip="https://www.screener.in/company/539594/consolidated/" xr:uid="{00000000-0004-0000-0000-000089010000}"/>
+    <hyperlink ref="B199" r:id="rId395" tooltip="https://www.screener.in/company/530617/" xr:uid="{00000000-0004-0000-0000-00008A010000}"/>
+    <hyperlink ref="M199" r:id="rId396" tooltip="https://www.screener.in/company/530617/" xr:uid="{00000000-0004-0000-0000-00008B010000}"/>
+    <hyperlink ref="B200" r:id="rId397" tooltip="https://www.screener.in/company/DANGEE/" xr:uid="{00000000-0004-0000-0000-00008C010000}"/>
+    <hyperlink ref="M200" r:id="rId398" tooltip="https://www.screener.in/company/DANGEE/" xr:uid="{00000000-0004-0000-0000-00008D010000}"/>
+    <hyperlink ref="B201" r:id="rId399" tooltip="https://www.screener.in/company/530217/" xr:uid="{00000000-0004-0000-0000-00008E010000}"/>
+    <hyperlink ref="M201" r:id="rId400" tooltip="https://www.screener.in/company/530217/" xr:uid="{00000000-0004-0000-0000-00008F010000}"/>
+    <hyperlink ref="B202" r:id="rId401" tooltip="https://www.screener.in/company/538520/" xr:uid="{00000000-0004-0000-0000-000090010000}"/>
+    <hyperlink ref="M202" r:id="rId402" tooltip="https://www.screener.in/company/538520/" xr:uid="{00000000-0004-0000-0000-000091010000}"/>
+    <hyperlink ref="B203" r:id="rId403" tooltip="https://www.screener.in/company/519500/" xr:uid="{00000000-0004-0000-0000-000092010000}"/>
+    <hyperlink ref="M203" r:id="rId404" tooltip="https://www.screener.in/company/519500/" xr:uid="{00000000-0004-0000-0000-000093010000}"/>
+    <hyperlink ref="B204" r:id="rId405" tooltip="https://www.screener.in/company/523105/" xr:uid="{00000000-0004-0000-0000-000094010000}"/>
+    <hyperlink ref="M204" r:id="rId406" tooltip="https://www.screener.in/company/523105/" xr:uid="{00000000-0004-0000-0000-000095010000}"/>
+    <hyperlink ref="B205" r:id="rId407" tooltip="https://www.screener.in/company/ROLLT/consolidated/" xr:uid="{00000000-0004-0000-0000-000096010000}"/>
+    <hyperlink ref="M205" r:id="rId408" tooltip="https://www.screener.in/company/ROLLT/consolidated/" xr:uid="{00000000-0004-0000-0000-000097010000}"/>
+    <hyperlink ref="B206" r:id="rId409" tooltip="https://www.screener.in/company/KAMOPAINTS/consolidated/" xr:uid="{00000000-0004-0000-0000-000098010000}"/>
+    <hyperlink ref="M206" r:id="rId410" tooltip="https://www.screener.in/company/KAMOPAINTS/consolidated/" xr:uid="{00000000-0004-0000-0000-000099010000}"/>
+    <hyperlink ref="B207" r:id="rId411" tooltip="https://www.screener.in/company/543579/" xr:uid="{00000000-0004-0000-0000-00009A010000}"/>
+    <hyperlink ref="M207" r:id="rId412" tooltip="https://www.screener.in/company/543579/" xr:uid="{00000000-0004-0000-0000-00009B010000}"/>
+    <hyperlink ref="B208" r:id="rId413" tooltip="https://www.screener.in/company/SIKKO/" xr:uid="{00000000-0004-0000-0000-00009C010000}"/>
+    <hyperlink ref="M208" r:id="rId414" tooltip="https://www.screener.in/company/SIKKO/" xr:uid="{00000000-0004-0000-0000-00009D010000}"/>
+    <hyperlink ref="B209" r:id="rId415" tooltip="https://www.screener.in/company/514165/consolidated/" xr:uid="{00000000-0004-0000-0000-00009E010000}"/>
+    <hyperlink ref="M209" r:id="rId416" tooltip="https://www.screener.in/company/514165/consolidated/" xr:uid="{00000000-0004-0000-0000-00009F010000}"/>
+    <hyperlink ref="B210" r:id="rId417" tooltip="https://www.screener.in/company/530027/" xr:uid="{00000000-0004-0000-0000-0000A0010000}"/>
+    <hyperlink ref="M210" r:id="rId418" tooltip="https://www.screener.in/company/530027/" xr:uid="{00000000-0004-0000-0000-0000A1010000}"/>
+    <hyperlink ref="B211" r:id="rId419" tooltip="https://www.screener.in/company/531739/consolidated/" xr:uid="{00000000-0004-0000-0000-0000A2010000}"/>
+    <hyperlink ref="M211" r:id="rId420" tooltip="https://www.screener.in/company/531739/consolidated/" xr:uid="{00000000-0004-0000-0000-0000A3010000}"/>
+    <hyperlink ref="B212" r:id="rId421" tooltip="https://www.screener.in/company/543499/" xr:uid="{00000000-0004-0000-0000-0000A4010000}"/>
+    <hyperlink ref="M212" r:id="rId422" tooltip="https://www.screener.in/company/543499/" xr:uid="{00000000-0004-0000-0000-0000A5010000}"/>
+    <hyperlink ref="B213" r:id="rId423" tooltip="https://www.screener.in/company/524238/" xr:uid="{00000000-0004-0000-0000-0000A6010000}"/>
+    <hyperlink ref="M213" r:id="rId424" tooltip="https://www.screener.in/company/524238/" xr:uid="{00000000-0004-0000-0000-0000A7010000}"/>
+    <hyperlink ref="B214" r:id="rId425" tooltip="https://www.screener.in/company/PILITA/" xr:uid="{00000000-0004-0000-0000-0000A8010000}"/>
+    <hyperlink ref="M214" r:id="rId426" tooltip="https://www.screener.in/company/PILITA/" xr:uid="{00000000-0004-0000-0000-0000A9010000}"/>
+    <hyperlink ref="B215" r:id="rId427" tooltip="https://www.screener.in/company/AVROIND/" xr:uid="{00000000-0004-0000-0000-0000AA010000}"/>
+    <hyperlink ref="M215" r:id="rId428" tooltip="https://www.screener.in/company/AVROIND/" xr:uid="{00000000-0004-0000-0000-0000AB010000}"/>
+    <hyperlink ref="B216" r:id="rId429" tooltip="https://www.screener.in/company/538817/consolidated/" xr:uid="{00000000-0004-0000-0000-0000AC010000}"/>
+    <hyperlink ref="M216" r:id="rId430" tooltip="https://www.screener.in/company/538817/consolidated/" xr:uid="{00000000-0004-0000-0000-0000AD010000}"/>
+    <hyperlink ref="B217" r:id="rId431" tooltip="https://www.screener.in/company/513337/consolidated/" xr:uid="{00000000-0004-0000-0000-0000AE010000}"/>
+    <hyperlink ref="M217" r:id="rId432" tooltip="https://www.screener.in/company/513337/consolidated/" xr:uid="{00000000-0004-0000-0000-0000AF010000}"/>
+    <hyperlink ref="B218" r:id="rId433" tooltip="https://www.screener.in/company/RTNPOWER/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B0010000}"/>
+    <hyperlink ref="M218" r:id="rId434" tooltip="https://www.screener.in/company/RTNPOWER/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B1010000}"/>
+    <hyperlink ref="B219" r:id="rId435" tooltip="https://www.screener.in/company/GREENPOWER/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B2010000}"/>
+    <hyperlink ref="M219" r:id="rId436" tooltip="https://www.screener.in/company/GREENPOWER/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B3010000}"/>
+    <hyperlink ref="B220" r:id="rId437" tooltip="https://www.screener.in/company/GVKPIL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B4010000}"/>
+    <hyperlink ref="M220" r:id="rId438" tooltip="https://www.screener.in/company/GVKPIL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B5010000}"/>
+    <hyperlink ref="B221" r:id="rId439" tooltip="https://www.screener.in/company/INDOWIND/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B6010000}"/>
+    <hyperlink ref="M221" r:id="rId440" tooltip="https://www.screener.in/company/INDOWIND/consolidated/" xr:uid="{00000000-0004-0000-0000-0000B7010000}"/>
+    <hyperlink ref="B222" r:id="rId441" tooltip="https://www.screener.in/company/500014/" xr:uid="{00000000-0004-0000-0000-0000B8010000}"/>
+    <hyperlink ref="M222" r:id="rId442" tooltip="https://www.screener.in/company/500014/" xr:uid="{00000000-0004-0000-0000-0000B9010000}"/>
+    <hyperlink ref="B223" r:id="rId443" tooltip="https://www.screener.in/company/INFOMEDIA/" xr:uid="{00000000-0004-0000-0000-0000BA010000}"/>
+    <hyperlink ref="M223" r:id="rId444" tooltip="https://www.screener.in/company/INFOMEDIA/" xr:uid="{00000000-0004-0000-0000-0000BB010000}"/>
+    <hyperlink ref="B224" r:id="rId445" tooltip="https://www.screener.in/company/526841/" xr:uid="{00000000-0004-0000-0000-0000BC010000}"/>
+    <hyperlink ref="M224" r:id="rId446" tooltip="https://www.screener.in/company/526841/" xr:uid="{00000000-0004-0000-0000-0000BD010000}"/>
+    <hyperlink ref="B225" r:id="rId447" tooltip="https://www.screener.in/company/KSHITIJPOL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000BE010000}"/>
+    <hyperlink ref="M225" r:id="rId448" tooltip="https://www.screener.in/company/KSHITIJPOL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000BF010000}"/>
+    <hyperlink ref="B226" r:id="rId449" tooltip="https://www.screener.in/company/LPDC/" xr:uid="{00000000-0004-0000-0000-0000C0010000}"/>
+    <hyperlink ref="M226" r:id="rId450" tooltip="https://www.screener.in/company/LPDC/" xr:uid="{00000000-0004-0000-0000-0000C1010000}"/>
+    <hyperlink ref="B227" r:id="rId451" tooltip="https://www.screener.in/company/530053/" xr:uid="{00000000-0004-0000-0000-0000C2010000}"/>
+    <hyperlink ref="M227" r:id="rId452" tooltip="https://www.screener.in/company/530053/" xr:uid="{00000000-0004-0000-0000-0000C3010000}"/>
+    <hyperlink ref="B228" r:id="rId453" tooltip="https://www.screener.in/company/543400/" xr:uid="{00000000-0004-0000-0000-0000C4010000}"/>
+    <hyperlink ref="M228" r:id="rId454" tooltip="https://www.screener.in/company/543400/" xr:uid="{00000000-0004-0000-0000-0000C5010000}"/>
+    <hyperlink ref="B229" r:id="rId455" tooltip="https://www.screener.in/company/UNITECH/consolidated/" xr:uid="{00000000-0004-0000-0000-0000C6010000}"/>
+    <hyperlink ref="M229" r:id="rId456" tooltip="https://www.screener.in/company/UNITECH/consolidated/" xr:uid="{00000000-0004-0000-0000-0000C7010000}"/>
+    <hyperlink ref="B230" r:id="rId457" tooltip="https://www.screener.in/company/NILAINFRA/consolidated/" xr:uid="{00000000-0004-0000-0000-0000C8010000}"/>
+    <hyperlink ref="M230" r:id="rId458" tooltip="https://www.screener.in/company/NILAINFRA/consolidated/" xr:uid="{00000000-0004-0000-0000-0000C9010000}"/>
+    <hyperlink ref="B231" r:id="rId459" tooltip="https://www.screener.in/company/HAMPTON/consolidated/" xr:uid="{00000000-0004-0000-0000-0000CA010000}"/>
+    <hyperlink ref="M231" r:id="rId460" tooltip="https://www.screener.in/company/HAMPTON/consolidated/" xr:uid="{00000000-0004-0000-0000-0000CB010000}"/>
+    <hyperlink ref="B232" r:id="rId461" tooltip="https://www.screener.in/company/PARSVNATH/consolidated/" xr:uid="{00000000-0004-0000-0000-0000CC010000}"/>
+    <hyperlink ref="M232" r:id="rId462" tooltip="https://www.screener.in/company/PARSVNATH/consolidated/" xr:uid="{00000000-0004-0000-0000-0000CD010000}"/>
+    <hyperlink ref="B233" r:id="rId463" tooltip="https://www.screener.in/company/531273/" xr:uid="{00000000-0004-0000-0000-0000CE010000}"/>
+    <hyperlink ref="M233" r:id="rId464" tooltip="https://www.screener.in/company/531273/" xr:uid="{00000000-0004-0000-0000-0000CF010000}"/>
+    <hyperlink ref="B234" r:id="rId465" tooltip="https://www.screener.in/company/NOIDATOLL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D0010000}"/>
+    <hyperlink ref="M234" r:id="rId466" tooltip="https://www.screener.in/company/NOIDATOLL/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D1010000}"/>
+    <hyperlink ref="B235" r:id="rId467" tooltip="https://www.screener.in/company/GAYAHWS/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D2010000}"/>
+    <hyperlink ref="M235" r:id="rId468" tooltip="https://www.screener.in/company/GAYAHWS/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D3010000}"/>
+    <hyperlink ref="B236" r:id="rId469" tooltip="https://www.screener.in/company/MEP/" xr:uid="{00000000-0004-0000-0000-0000D4010000}"/>
+    <hyperlink ref="M236" r:id="rId470" tooltip="https://www.screener.in/company/MEP/" xr:uid="{00000000-0004-0000-0000-0000D5010000}"/>
+    <hyperlink ref="B237" r:id="rId471" tooltip="https://www.screener.in/company/526795/" xr:uid="{00000000-0004-0000-0000-0000D6010000}"/>
+    <hyperlink ref="M237" r:id="rId472" tooltip="https://www.screener.in/company/526795/" xr:uid="{00000000-0004-0000-0000-0000D7010000}"/>
+    <hyperlink ref="B238" r:id="rId473" tooltip="https://www.screener.in/company/AVANCE/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D8010000}"/>
+    <hyperlink ref="M238" r:id="rId474" tooltip="https://www.screener.in/company/AVANCE/consolidated/" xr:uid="{00000000-0004-0000-0000-0000D9010000}"/>
+    <hyperlink ref="B239" r:id="rId475" tooltip="https://www.screener.in/company/512093/consolidated/" xr:uid="{00000000-0004-0000-0000-0000DA010000}"/>
+    <hyperlink ref="M239" r:id="rId476" tooltip="https://www.screener.in/company/512093/consolidated/" xr:uid="{00000000-0004-0000-0000-0000DB010000}"/>
+    <hyperlink ref="B240" r:id="rId477" tooltip="https://www.screener.in/company/PRAXIS/" xr:uid="{00000000-0004-0000-0000-0000DC010000}"/>
+    <hyperlink ref="M240" r:id="rId478" tooltip="https://www.screener.in/company/PRAXIS/" xr:uid="{00000000-0004-0000-0000-0000DD010000}"/>
+    <hyperlink ref="B241" r:id="rId479" tooltip="https://www.screener.in/company/540615/" xr:uid="{00000000-0004-0000-0000-0000DE010000}"/>
+    <hyperlink ref="M241" r:id="rId480" tooltip="https://www.screener.in/company/540615/" xr:uid="{00000000-0004-0000-0000-0000DF010000}"/>
+    <hyperlink ref="B242" r:id="rId481" tooltip="https://www.screener.in/company/VIKASECO/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E0010000}"/>
+    <hyperlink ref="M242" r:id="rId482" tooltip="https://www.screener.in/company/VIKASECO/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E1010000}"/>
+    <hyperlink ref="B243" r:id="rId483" tooltip="https://www.screener.in/company/SUNDARAM/" xr:uid="{00000000-0004-0000-0000-0000E2010000}"/>
+    <hyperlink ref="M243" r:id="rId484" tooltip="https://www.screener.in/company/SUNDARAM/" xr:uid="{00000000-0004-0000-0000-0000E3010000}"/>
+    <hyperlink ref="B244" r:id="rId485" tooltip="https://www.screener.in/company/539228/" xr:uid="{00000000-0004-0000-0000-0000E4010000}"/>
+    <hyperlink ref="M244" r:id="rId486" tooltip="https://www.screener.in/company/539228/" xr:uid="{00000000-0004-0000-0000-0000E5010000}"/>
+    <hyperlink ref="B245" r:id="rId487" tooltip="https://www.screener.in/company/VASA/" xr:uid="{00000000-0004-0000-0000-0000E6010000}"/>
+    <hyperlink ref="M245" r:id="rId488" tooltip="https://www.screener.in/company/VASA/" xr:uid="{00000000-0004-0000-0000-0000E7010000}"/>
+    <hyperlink ref="B246" r:id="rId489" tooltip="https://www.screener.in/company/INVENTURE/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E8010000}"/>
+    <hyperlink ref="M246" r:id="rId490" tooltip="https://www.screener.in/company/INVENTURE/consolidated/" xr:uid="{00000000-0004-0000-0000-0000E9010000}"/>
+    <hyperlink ref="B247" r:id="rId491" tooltip="https://www.screener.in/company/535431/" xr:uid="{00000000-0004-0000-0000-0000EA010000}"/>
+    <hyperlink ref="M247" r:id="rId492" tooltip="https://www.screener.in/company/535431/" xr:uid="{00000000-0004-0000-0000-0000EB010000}"/>
+    <hyperlink ref="B248" r:id="rId493" tooltip="https://www.screener.in/company/VISHWARAJ/" xr:uid="{00000000-0004-0000-0000-0000EC010000}"/>
+    <hyperlink ref="M248" r:id="rId494" tooltip="https://www.screener.in/company/VISHWARAJ/" xr:uid="{00000000-0004-0000-0000-0000ED010000}"/>
+    <hyperlink ref="B249" r:id="rId495" tooltip="https://www.screener.in/company/541347/" xr:uid="{00000000-0004-0000-0000-0000EE010000}"/>
+    <hyperlink ref="M249" r:id="rId496" tooltip="https://www.screener.in/company/541347/" xr:uid="{00000000-0004-0000-0000-0000EF010000}"/>
+    <hyperlink ref="B250" r:id="rId497" tooltip="https://www.screener.in/company/532183/" xr:uid="{00000000-0004-0000-0000-0000F0010000}"/>
+    <hyperlink ref="M250" r:id="rId498" tooltip="https://www.screener.in/company/532183/" xr:uid="{00000000-0004-0000-0000-0000F1010000}"/>
+    <hyperlink ref="B251" r:id="rId499" tooltip="https://www.screener.in/company/SIMBHALS/consolidated/" xr:uid="{00000000-0004-0000-0000-0000F2010000}"/>
+    <hyperlink ref="M251" r:id="rId500" tooltip="https://www.screener.in/company/SIMBHALS/consolidated/" xr:uid="{00000000-0004-0000-0000-0000F3010000}"/>
+    <hyperlink ref="B252" r:id="rId501" tooltip="https://www.screener.in/company/537709/" xr:uid="{00000000-0004-0000-0000-0000F4010000}"/>
+    <hyperlink ref="M252" r:id="rId502" tooltip="https://www.screener.in/company/537709/" xr:uid="{00000000-0004-0000-0000-0000F5010000}"/>
+    <hyperlink ref="B253" r:id="rId503" tooltip="https://www.screener.in/company/AKSHOPTFBR/consolidated/" xr:uid="{00000000-0004-0000-0000-0000F6010000}"/>
+    <hyperlink ref="M253" r:id="rId504" tooltip="https://www.screener.in/company/AKSHOPTFBR/consolidated/" xr:uid="{00000000-0004-0000-0000-0000F7010000}"/>
+    <hyperlink ref="B254" r:id="rId505" tooltip="https://www.screener.in/company/532975/" xr:uid="{00000000-0004-0000-0000-0000F8010000}"/>
+    <hyperlink ref="M254" r:id="rId506" tooltip="https://www.screener.in/company/532975/" xr:uid="{00000000-0004-0000-0000-0000F9010000}"/>
+    <hyperlink ref="B255" r:id="rId507" tooltip="https://www.screener.in/company/RCOM/consolidated/" xr:uid="{00000000-0004-0000-0000-0000FA010000}"/>
+    <hyperlink ref="M255" r:id="rId508" tooltip="https://www.screener.in/company/RCOM/consolidated/" xr:uid="{00000000-0004-0000-0000-0000FB010000}"/>
+    <hyperlink ref="B256" r:id="rId509" tooltip="https://www.screener.in/company/511116/" xr:uid="{00000000-0004-0000-0000-0000FC010000}"/>
+    <hyperlink ref="M256" r:id="rId510" tooltip="https://www.screener.in/company/511116/" xr:uid="{00000000-0004-0000-0000-0000FD010000}"/>
+    <hyperlink ref="B257" r:id="rId511" tooltip="https://www.screener.in/company/538674/" xr:uid="{00000000-0004-0000-0000-0000FE010000}"/>
+    <hyperlink ref="M257" r:id="rId512" tooltip="https://www.screener.in/company/538674/" xr:uid="{00000000-0004-0000-0000-0000FF010000}"/>
+    <hyperlink ref="B258" r:id="rId513" tooltip="https://www.screener.in/company/GTLINFRA/" xr:uid="{00000000-0004-0000-0000-000000020000}"/>
+    <hyperlink ref="M258" r:id="rId514" tooltip="https://www.screener.in/company/GTLINFRA/" xr:uid="{00000000-0004-0000-0000-000001020000}"/>
+    <hyperlink ref="B259" r:id="rId515" tooltip="https://www.screener.in/company/EASEMYTRIP/consolidated/" xr:uid="{00000000-0004-0000-0000-000002020000}"/>
+    <hyperlink ref="M259" r:id="rId516" tooltip="https://www.screener.in/company/EASEMYTRIP/consolidated/" xr:uid="{00000000-0004-0000-0000-000003020000}"/>
+    <hyperlink ref="B260" r:id="rId517" tooltip="https://www.screener.in/company/544242/" xr:uid="{00000000-0004-0000-0000-000004020000}"/>
+    <hyperlink ref="M260" r:id="rId518" tooltip="https://www.screener.in/company/544242/" xr:uid="{00000000-0004-0000-0000-000005020000}"/>
+    <hyperlink ref="B261" r:id="rId519" tooltip="https://www.screener.in/company/543541/" xr:uid="{00000000-0004-0000-0000-000006020000}"/>
+    <hyperlink ref="M261" r:id="rId520" tooltip="https://www.screener.in/company/543541/" xr:uid="{00000000-0004-0000-0000-000007020000}"/>
+    <hyperlink ref="B262" r:id="rId521" tooltip="https://www.screener.in/company/524444/consolidated/" xr:uid="{00000000-0004-0000-0000-000008020000}"/>
+    <hyperlink ref="M262" r:id="rId522" tooltip="https://www.screener.in/company/524444/consolidated/" xr:uid="{00000000-0004-0000-0000-000009020000}"/>
+    <hyperlink ref="B263" r:id="rId523" tooltip="https://www.screener.in/company/542012/" xr:uid="{00000000-0004-0000-0000-00000A020000}"/>
+    <hyperlink ref="M263" r:id="rId524" tooltip="https://www.screener.in/company/542012/" xr:uid="{00000000-0004-0000-0000-00000B020000}"/>
+    <hyperlink ref="B264" r:id="rId525" tooltip="https://www.screener.in/company/539800/" xr:uid="{00000000-0004-0000-0000-00000C020000}"/>
+    <hyperlink ref="M264" r:id="rId526" tooltip="https://www.screener.in/company/539800/" xr:uid="{00000000-0004-0000-0000-00000D020000}"/>
+    <hyperlink ref="B265" r:id="rId527" tooltip="https://www.screener.in/company/543798/" xr:uid="{00000000-0004-0000-0000-00000E020000}"/>
+    <hyperlink ref="M265" r:id="rId528" tooltip="https://www.screener.in/company/543798/" xr:uid="{00000000-0004-0000-0000-00000F020000}"/>
+    <hyperlink ref="B266" r:id="rId529" tooltip="https://www.screener.in/company/540492/" xr:uid="{00000000-0004-0000-0000-000010020000}"/>
+    <hyperlink ref="M266" r:id="rId530" tooltip="https://www.screener.in/company/540492/" xr:uid="{00000000-0004-0000-0000-000011020000}"/>
+    <hyperlink ref="B267" r:id="rId531" tooltip="https://www.screener.in/company/HEADSUP/" xr:uid="{00000000-0004-0000-0000-000012020000}"/>
+    <hyperlink ref="M267" r:id="rId532" tooltip="https://www.screener.in/company/HEADSUP/" xr:uid="{00000000-0004-0000-0000-000013020000}"/>
+    <hyperlink ref="B268" r:id="rId533" tooltip="https://www.screener.in/company/542206/" xr:uid="{00000000-0004-0000-0000-000014020000}"/>
+    <hyperlink ref="M268" r:id="rId534" tooltip="https://www.screener.in/company/542206/" xr:uid="{00000000-0004-0000-0000-000015020000}"/>
+    <hyperlink ref="B269" r:id="rId535" tooltip="https://www.screener.in/company/540717/consolidated/" xr:uid="{00000000-0004-0000-0000-000016020000}"/>
+    <hyperlink ref="M269" r:id="rId536" tooltip="https://www.screener.in/company/540717/consolidated/" xr:uid="{00000000-0004-0000-0000-000017020000}"/>
+    <hyperlink ref="B270" r:id="rId537" tooltip="https://www.screener.in/company/SAKUMA/consolidated/" xr:uid="{00000000-0004-0000-0000-000018020000}"/>
+    <hyperlink ref="M270" r:id="rId538" tooltip="https://www.screener.in/company/SAKUMA/consolidated/" xr:uid="{00000000-0004-0000-0000-000019020000}"/>
+    <hyperlink ref="B271" r:id="rId539" tooltip="https://www.screener.in/company/VIKASLIFE/consolidated/" xr:uid="{00000000-0004-0000-0000-00001A020000}"/>
+    <hyperlink ref="M271" r:id="rId540" tooltip="https://www.screener.in/company/VIKASLIFE/consolidated/" xr:uid="{00000000-0004-0000-0000-00001B020000}"/>
+    <hyperlink ref="B272" r:id="rId541" tooltip="https://www.screener.in/company/SPCENET/consolidated/" xr:uid="{00000000-0004-0000-0000-00001C020000}"/>
+    <hyperlink ref="M272" r:id="rId542" tooltip="https://www.screener.in/company/SPCENET/consolidated/" xr:uid="{00000000-0004-0000-0000-00001D020000}"/>
+    <hyperlink ref="B273" r:id="rId543" tooltip="https://www.screener.in/company/ESSENTIA/consolidated/" xr:uid="{00000000-0004-0000-0000-00001E020000}"/>
+    <hyperlink ref="M273" r:id="rId544" tooltip="https://www.screener.in/company/ESSENTIA/consolidated/" xr:uid="{00000000-0004-0000-0000-00001F020000}"/>
+    <hyperlink ref="B274" r:id="rId545" tooltip="https://www.screener.in/company/LANDSMILL/consolidated/" xr:uid="{00000000-0004-0000-0000-000020020000}"/>
+    <hyperlink ref="M274" r:id="rId546" tooltip="https://www.screener.in/company/LANDSMILL/consolidated/" xr:uid="{00000000-0004-0000-0000-000021020000}"/>
+    <hyperlink ref="B275" r:id="rId547" tooltip="https://www.screener.in/company/HATHWAY/consolidated/" xr:uid="{00000000-0004-0000-0000-000022020000}"/>
+    <hyperlink ref="M275" r:id="rId548" tooltip="https://www.screener.in/company/HATHWAY/consolidated/" xr:uid="{00000000-0004-0000-0000-000023020000}"/>
+    <hyperlink ref="B276" r:id="rId549" tooltip="https://www.screener.in/company/ZEEMEDIA/consolidated/" xr:uid="{00000000-0004-0000-0000-000024020000}"/>
+    <hyperlink ref="M276" r:id="rId550" tooltip="https://www.screener.in/company/ZEEMEDIA/consolidated/" xr:uid="{00000000-0004-0000-0000-000025020000}"/>
+    <hyperlink ref="B277" r:id="rId551" tooltip="https://www.screener.in/company/DISHTV/consolidated/" xr:uid="{00000000-0004-0000-0000-000026020000}"/>
+    <hyperlink ref="M277" r:id="rId552" tooltip="https://www.screener.in/company/DISHTV/consolidated/" xr:uid="{00000000-0004-0000-0000-000027020000}"/>
+    <hyperlink ref="B278" r:id="rId553" tooltip="https://www.screener.in/company/BAGFILMS/consolidated/" xr:uid="{00000000-0004-0000-0000-000028020000}"/>
+    <hyperlink ref="M278" r:id="rId554" tooltip="https://www.screener.in/company/BAGFILMS/consolidated/" xr:uid="{00000000-0004-0000-0000-000029020000}"/>
+    <hyperlink ref="B279" r:id="rId555" tooltip="https://www.screener.in/company/SITINET/consolidated/" xr:uid="{00000000-0004-0000-0000-00002A020000}"/>
+    <hyperlink ref="M279" r:id="rId556" tooltip="https://www.screener.in/company/SITINET/consolidated/" xr:uid="{00000000-0004-0000-0000-00002B020000}"/>
+    <hyperlink ref="B280" r:id="rId557" tooltip="https://www.screener.in/company/540821/" xr:uid="{00000000-0004-0000-0000-00002C020000}"/>
+    <hyperlink ref="M280" r:id="rId558" tooltip="https://www.screener.in/company/540821/" xr:uid="{00000000-0004-0000-0000-00002D020000}"/>
+    <hyperlink ref="B281" r:id="rId559" tooltip="https://www.screener.in/company/521062/" xr:uid="{00000000-0004-0000-0000-00002E020000}"/>
+    <hyperlink ref="M281" r:id="rId560" tooltip="https://www.screener.in/company/521062/" xr:uid="{00000000-0004-0000-0000-00002F020000}"/>
+    <hyperlink ref="B282" r:id="rId561" tooltip="https://www.screener.in/company/TVVISION/consolidated/" xr:uid="{00000000-0004-0000-0000-000030020000}"/>
+    <hyperlink ref="M282" r:id="rId562" tooltip="https://www.screener.in/company/TVVISION/consolidated/" xr:uid="{00000000-0004-0000-0000-000031020000}"/>
+    <hyperlink ref="B283" r:id="rId563" tooltip="https://www.screener.in/company/ORTEL/" xr:uid="{00000000-0004-0000-0000-000032020000}"/>
+    <hyperlink ref="M283" r:id="rId564" tooltip="https://www.screener.in/company/ORTEL/" xr:uid="{00000000-0004-0000-0000-000033020000}"/>
+    <hyperlink ref="B284" r:id="rId565" tooltip="https://www.screener.in/company/533268/consolidated/" xr:uid="{00000000-0004-0000-0000-000034020000}"/>
+    <hyperlink ref="M284" r:id="rId566" tooltip="https://www.screener.in/company/533268/consolidated/" xr:uid="{00000000-0004-0000-0000-000035020000}"/>
+    <hyperlink ref="B285" r:id="rId567" tooltip="https://www.screener.in/company/539040/" xr:uid="{00000000-0004-0000-0000-000036020000}"/>
+    <hyperlink ref="M285" r:id="rId568" tooltip="https://www.screener.in/company/539040/" xr:uid="{00000000-0004-0000-0000-000037020000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="9" width="12" customWidth="1"/>
-    <col min="10" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="30" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>2225</v>
-      </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:M1"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:M2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>